<commit_message>
Cons file: add monthly CAPEX 2027 sheet and 2026 summary in new Commercial margin logic
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TjyVtBMeKRjjZMJmWM6RZp
</commit_message>
<xml_diff>
--- a/Adtech_BU2027_для_конс.xlsx
+++ b/Adtech_BU2027_для_конс.xlsx
@@ -9,6 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Свод BU2027" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BU2027 расчёт" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CAPEX BU2027" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Свод 2026 (новая логика)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026 расчёт" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -112,7 +115,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -159,6 +162,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
         <bgColor rgb="FFDAE3F3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.7999816888943144"/>
       </patternFill>
     </fill>
   </fills>
@@ -230,7 +238,7 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -507,6 +515,9 @@
     </xf>
     <xf numFmtId="167" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -2532,14 +2543,14 @@
       </c>
       <c r="N6" s="89">
         <f>SUM(B6:M6)</f>
-        <v/>
+        <v>7696.23419752104</v>
       </c>
       <c r="O6" s="89" t="n">
         <v>6195.4</v>
       </c>
       <c r="P6" s="89">
         <f>N6-O6</f>
-        <v/>
+        <v>1500.83419752104</v>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="48">
@@ -2586,14 +2597,14 @@
       </c>
       <c r="N7" s="89">
         <f>SUM(B7:M7)</f>
-        <v/>
+        <v>1600</v>
       </c>
       <c r="O7" s="89" t="n">
         <v>986.999999999999</v>
       </c>
       <c r="P7" s="89">
         <f>N7-O7</f>
-        <v/>
+        <v>613.000000000001</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="48">
@@ -2640,14 +2651,14 @@
       </c>
       <c r="N8" s="89">
         <f>SUM(B8:M8)</f>
-        <v/>
+        <v>187</v>
       </c>
       <c r="O8" s="89" t="n">
         <v>102.4</v>
       </c>
       <c r="P8" s="89">
         <f>N8-O8</f>
-        <v/>
+        <v>84.6</v>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="48">
@@ -2694,14 +2705,14 @@
       </c>
       <c r="N9" s="89">
         <f>SUM(B9:M9)</f>
-        <v/>
+        <v>4019.49176286191</v>
       </c>
       <c r="O9" s="89" t="n">
         <v>2446.0892363</v>
       </c>
       <c r="P9" s="89">
         <f>N9-O9</f>
-        <v/>
+        <v>1573.40252656191</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="48">
@@ -2748,14 +2759,14 @@
       </c>
       <c r="N10" s="89">
         <f>SUM(B10:M10)</f>
-        <v/>
+        <v>213.3</v>
       </c>
       <c r="O10" s="89" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="89">
         <f>N10-O10</f>
-        <v/>
+        <v>213.3</v>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="48">
@@ -2802,14 +2813,14 @@
       </c>
       <c r="N11" s="89">
         <f>SUM(B11:M11)</f>
-        <v/>
+        <v>850.209144949859</v>
       </c>
       <c r="O11" s="89" t="n">
         <v>592.5599999999999</v>
       </c>
       <c r="P11" s="89">
         <f>N11-O11</f>
-        <v/>
+        <v>257.649144949859</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="48">
@@ -2820,63 +2831,63 @@
       </c>
       <c r="B12" s="90">
         <f>SUM(B6:B11)</f>
-        <v/>
+        <v>291.325773985418</v>
       </c>
       <c r="C12" s="90">
         <f>SUM(C6:C11)</f>
-        <v/>
+        <v>728.318901125052</v>
       </c>
       <c r="D12" s="90">
         <f>SUM(D6:D11)</f>
-        <v/>
+        <v>1019.64020894896</v>
       </c>
       <c r="E12" s="90">
         <f>SUM(E6:E11)</f>
-        <v/>
+        <v>1019.62681046444</v>
       </c>
       <c r="F12" s="90">
         <f>SUM(F6:F11)</f>
-        <v/>
+        <v>1019.64020894896</v>
       </c>
       <c r="G12" s="90">
         <f>SUM(G6:G11)</f>
-        <v/>
+        <v>1019.64020894896</v>
       </c>
       <c r="H12" s="90">
         <f>SUM(H6:H11)</f>
-        <v/>
+        <v>1019.64020894896</v>
       </c>
       <c r="I12" s="90">
         <f>SUM(I6:I11)</f>
-        <v/>
+        <v>1165.28076513413</v>
       </c>
       <c r="J12" s="90">
         <f>SUM(J6:J11)</f>
-        <v/>
+        <v>1165.28076513413</v>
       </c>
       <c r="K12" s="90">
         <f>SUM(K6:K11)</f>
-        <v/>
+        <v>1602.2917569198</v>
       </c>
       <c r="L12" s="90">
         <f>SUM(L6:L11)</f>
-        <v/>
+        <v>2039.28041789792</v>
       </c>
       <c r="M12" s="90">
         <f>SUM(M6:M11)</f>
-        <v/>
+        <v>2476.26907887606</v>
       </c>
       <c r="N12" s="90">
         <f>SUM(N6:N11)</f>
-        <v/>
+        <v>14566.2351053328</v>
       </c>
       <c r="O12" s="90">
         <f>SUM(O6:O11)</f>
-        <v/>
+        <v>10323.4492363</v>
       </c>
       <c r="P12" s="90">
         <f>SUM(P6:P11)</f>
-        <v/>
+        <v>4242.78586903281</v>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="48">
@@ -2926,55 +2937,55 @@
       </c>
       <c r="B15" s="89">
         <f>IF($N6=0,0,$P6*B6/$N6)</f>
-        <v/>
+        <v>30.0166839504208</v>
       </c>
       <c r="C15" s="89">
         <f>IF($N6=0,0,$P6*C6/$N6)</f>
-        <v/>
+        <v>75.0417098760519</v>
       </c>
       <c r="D15" s="89">
         <f>IF($N6=0,0,$P6*D6/$N6)</f>
-        <v/>
+        <v>105.058393826473</v>
       </c>
       <c r="E15" s="89">
         <f>IF($N6=0,0,$P6*E6/$N6)</f>
-        <v/>
+        <v>105.058393826472</v>
       </c>
       <c r="F15" s="89">
         <f>IF($N6=0,0,$P6*F6/$N6)</f>
-        <v/>
+        <v>105.058393826473</v>
       </c>
       <c r="G15" s="89">
         <f>IF($N6=0,0,$P6*G6/$N6)</f>
-        <v/>
+        <v>105.058393826473</v>
       </c>
       <c r="H15" s="89">
         <f>IF($N6=0,0,$P6*H6/$N6)</f>
-        <v/>
+        <v>105.058393826473</v>
       </c>
       <c r="I15" s="89">
         <f>IF($N6=0,0,$P6*I6/$N6)</f>
-        <v/>
+        <v>120.066735801683</v>
       </c>
       <c r="J15" s="89">
         <f>IF($N6=0,0,$P6*J6/$N6)</f>
-        <v/>
+        <v>120.066735801683</v>
       </c>
       <c r="K15" s="89">
         <f>IF($N6=0,0,$P6*K6/$N6)</f>
-        <v/>
+        <v>165.091761727314</v>
       </c>
       <c r="L15" s="89">
         <f>IF($N6=0,0,$P6*L6/$N6)</f>
-        <v/>
+        <v>210.116787652944</v>
       </c>
       <c r="M15" s="89">
         <f>IF($N6=0,0,$P6*M6/$N6)</f>
-        <v/>
+        <v>255.141813578577</v>
       </c>
       <c r="N15" s="89">
         <f>SUM(B15:M15)</f>
-        <v/>
+        <v>1500.83419752104</v>
       </c>
       <c r="O15" s="89" t="n"/>
       <c r="P15" s="89" t="n"/>
@@ -2987,55 +2998,55 @@
       </c>
       <c r="B16" s="89">
         <f>IF($N7=0,0,$P7*B7/$N7)</f>
-        <v/>
+        <v>12.26</v>
       </c>
       <c r="C16" s="89">
         <f>IF($N7=0,0,$P7*C7/$N7)</f>
-        <v/>
+        <v>30.65</v>
       </c>
       <c r="D16" s="89">
         <f>IF($N7=0,0,$P7*D7/$N7)</f>
-        <v/>
+        <v>42.9100000000001</v>
       </c>
       <c r="E16" s="89">
         <f>IF($N7=0,0,$P7*E7/$N7)</f>
-        <v/>
+        <v>42.9100000000001</v>
       </c>
       <c r="F16" s="89">
         <f>IF($N7=0,0,$P7*F7/$N7)</f>
-        <v/>
+        <v>42.9100000000001</v>
       </c>
       <c r="G16" s="89">
         <f>IF($N7=0,0,$P7*G7/$N7)</f>
-        <v/>
+        <v>42.9100000000001</v>
       </c>
       <c r="H16" s="89">
         <f>IF($N7=0,0,$P7*H7/$N7)</f>
-        <v/>
+        <v>42.9100000000001</v>
       </c>
       <c r="I16" s="89">
         <f>IF($N7=0,0,$P7*I7/$N7)</f>
-        <v/>
+        <v>49.0400000000001</v>
       </c>
       <c r="J16" s="89">
         <f>IF($N7=0,0,$P7*J7/$N7)</f>
-        <v/>
+        <v>49.0400000000001</v>
       </c>
       <c r="K16" s="89">
         <f>IF($N7=0,0,$P7*K7/$N7)</f>
-        <v/>
+        <v>67.4300000000001</v>
       </c>
       <c r="L16" s="89">
         <f>IF($N7=0,0,$P7*L7/$N7)</f>
-        <v/>
+        <v>85.8200000000002</v>
       </c>
       <c r="M16" s="89">
         <f>IF($N7=0,0,$P7*M7/$N7)</f>
-        <v/>
+        <v>104.21</v>
       </c>
       <c r="N16" s="89">
         <f>SUM(B16:M16)</f>
-        <v/>
+        <v>613.000000000001</v>
       </c>
       <c r="O16" s="89" t="n"/>
       <c r="P16" s="89" t="n"/>
@@ -3048,55 +3059,55 @@
       </c>
       <c r="B17" s="89">
         <f>IF($N8=0,0,$P8*B8/$N8)</f>
-        <v/>
+        <v>1.692</v>
       </c>
       <c r="C17" s="89">
         <f>IF($N8=0,0,$P8*C8/$N8)</f>
-        <v/>
+        <v>4.23</v>
       </c>
       <c r="D17" s="89">
         <f>IF($N8=0,0,$P8*D8/$N8)</f>
-        <v/>
+        <v>5.922</v>
       </c>
       <c r="E17" s="89">
         <f>IF($N8=0,0,$P8*E8/$N8)</f>
-        <v/>
+        <v>5.922</v>
       </c>
       <c r="F17" s="89">
         <f>IF($N8=0,0,$P8*F8/$N8)</f>
-        <v/>
+        <v>5.922</v>
       </c>
       <c r="G17" s="89">
         <f>IF($N8=0,0,$P8*G8/$N8)</f>
-        <v/>
+        <v>5.922</v>
       </c>
       <c r="H17" s="89">
         <f>IF($N8=0,0,$P8*H8/$N8)</f>
-        <v/>
+        <v>5.922</v>
       </c>
       <c r="I17" s="89">
         <f>IF($N8=0,0,$P8*I8/$N8)</f>
-        <v/>
+        <v>6.768</v>
       </c>
       <c r="J17" s="89">
         <f>IF($N8=0,0,$P8*J8/$N8)</f>
-        <v/>
+        <v>6.768</v>
       </c>
       <c r="K17" s="89">
         <f>IF($N8=0,0,$P8*K8/$N8)</f>
-        <v/>
+        <v>9.306</v>
       </c>
       <c r="L17" s="89">
         <f>IF($N8=0,0,$P8*L8/$N8)</f>
-        <v/>
+        <v>11.844</v>
       </c>
       <c r="M17" s="89">
         <f>IF($N8=0,0,$P8*M8/$N8)</f>
-        <v/>
+        <v>14.382</v>
       </c>
       <c r="N17" s="89">
         <f>SUM(B17:M17)</f>
-        <v/>
+        <v>84.6</v>
       </c>
       <c r="O17" s="89" t="n"/>
       <c r="P17" s="89" t="n"/>
@@ -3109,55 +3120,55 @@
       </c>
       <c r="B18" s="89">
         <f>IF($N9=0,0,$P9*B9/$N9)</f>
-        <v/>
+        <v>31.4684701108396</v>
       </c>
       <c r="C18" s="89">
         <f>IF($N9=0,0,$P9*C9/$N9)</f>
-        <v/>
+        <v>78.6729235254384</v>
       </c>
       <c r="D18" s="89">
         <f>IF($N9=0,0,$P9*D9/$N9)</f>
-        <v/>
+        <v>110.139645387939</v>
       </c>
       <c r="E18" s="89">
         <f>IF($N9=0,0,$P9*E9/$N9)</f>
-        <v/>
+        <v>110.13440064292</v>
       </c>
       <c r="F18" s="89">
         <f>IF($N9=0,0,$P9*F9/$N9)</f>
-        <v/>
+        <v>110.139645387939</v>
       </c>
       <c r="G18" s="89">
         <f>IF($N9=0,0,$P9*G9/$N9)</f>
-        <v/>
+        <v>110.139645387939</v>
       </c>
       <c r="H18" s="89">
         <f>IF($N9=0,0,$P9*H9/$N9)</f>
-        <v/>
+        <v>110.139645387939</v>
       </c>
       <c r="I18" s="89">
         <f>IF($N9=0,0,$P9*I9/$N9)</f>
-        <v/>
+        <v>125.865139201661</v>
       </c>
       <c r="J18" s="89">
         <f>IF($N9=0,0,$P9*J9/$N9)</f>
-        <v/>
+        <v>125.865139201661</v>
       </c>
       <c r="K18" s="89">
         <f>IF($N9=0,0,$P9*K9/$N9)</f>
-        <v/>
+        <v>173.076585609618</v>
       </c>
       <c r="L18" s="89">
         <f>IF($N9=0,0,$P9*L9/$N9)</f>
-        <v/>
+        <v>220.279290775877</v>
       </c>
       <c r="M18" s="89">
         <f>IF($N9=0,0,$P9*M9/$N9)</f>
-        <v/>
+        <v>267.481995942137</v>
       </c>
       <c r="N18" s="89">
         <f>SUM(B18:M18)</f>
-        <v/>
+        <v>1573.40252656191</v>
       </c>
       <c r="O18" s="89" t="n"/>
       <c r="P18" s="89" t="n"/>
@@ -3170,55 +3181,55 @@
       </c>
       <c r="B19" s="89">
         <f>IF($N10=0,0,$P10*B10/$N10)</f>
-        <v/>
+        <v>4.266</v>
       </c>
       <c r="C19" s="89">
         <f>IF($N10=0,0,$P10*C10/$N10)</f>
-        <v/>
+        <v>10.665</v>
       </c>
       <c r="D19" s="89">
         <f>IF($N10=0,0,$P10*D10/$N10)</f>
-        <v/>
+        <v>14.931</v>
       </c>
       <c r="E19" s="89">
         <f>IF($N10=0,0,$P10*E10/$N10)</f>
-        <v/>
+        <v>14.931</v>
       </c>
       <c r="F19" s="89">
         <f>IF($N10=0,0,$P10*F10/$N10)</f>
-        <v/>
+        <v>14.931</v>
       </c>
       <c r="G19" s="89">
         <f>IF($N10=0,0,$P10*G10/$N10)</f>
-        <v/>
+        <v>14.931</v>
       </c>
       <c r="H19" s="89">
         <f>IF($N10=0,0,$P10*H10/$N10)</f>
-        <v/>
+        <v>14.931</v>
       </c>
       <c r="I19" s="89">
         <f>IF($N10=0,0,$P10*I10/$N10)</f>
-        <v/>
+        <v>17.064</v>
       </c>
       <c r="J19" s="89">
         <f>IF($N10=0,0,$P10*J10/$N10)</f>
-        <v/>
+        <v>17.064</v>
       </c>
       <c r="K19" s="89">
         <f>IF($N10=0,0,$P10*K10/$N10)</f>
-        <v/>
+        <v>23.4630000000001</v>
       </c>
       <c r="L19" s="89">
         <f>IF($N10=0,0,$P10*L10/$N10)</f>
-        <v/>
+        <v>29.862</v>
       </c>
       <c r="M19" s="89">
         <f>IF($N10=0,0,$P10*M10/$N10)</f>
-        <v/>
+        <v>36.2609999999999</v>
       </c>
       <c r="N19" s="89">
         <f>SUM(B19:M19)</f>
-        <v/>
+        <v>213.3</v>
       </c>
       <c r="O19" s="89" t="n"/>
       <c r="P19" s="89" t="n"/>
@@ -3231,55 +3242,55 @@
       </c>
       <c r="B20" s="89">
         <f>IF($N11=0,0,$P11*B11/$N11)</f>
-        <v/>
+        <v>5.15298289899719</v>
       </c>
       <c r="C20" s="89">
         <f>IF($N11=0,0,$P11*C11/$N11)</f>
-        <v/>
+        <v>12.882457247493</v>
       </c>
       <c r="D20" s="89">
         <f>IF($N11=0,0,$P11*D11/$N11)</f>
-        <v/>
+        <v>18.0354401464902</v>
       </c>
       <c r="E20" s="89">
         <f>IF($N11=0,0,$P11*E11/$N11)</f>
-        <v/>
+        <v>18.0354401464902</v>
       </c>
       <c r="F20" s="89">
         <f>IF($N11=0,0,$P11*F11/$N11)</f>
-        <v/>
+        <v>18.0354401464902</v>
       </c>
       <c r="G20" s="89">
         <f>IF($N11=0,0,$P11*G11/$N11)</f>
-        <v/>
+        <v>18.0354401464902</v>
       </c>
       <c r="H20" s="89">
         <f>IF($N11=0,0,$P11*H11/$N11)</f>
-        <v/>
+        <v>18.0354401464902</v>
       </c>
       <c r="I20" s="89">
         <f>IF($N11=0,0,$P11*I11/$N11)</f>
-        <v/>
+        <v>20.6119315959888</v>
       </c>
       <c r="J20" s="89">
         <f>IF($N11=0,0,$P11*J11/$N11)</f>
-        <v/>
+        <v>20.6119315959888</v>
       </c>
       <c r="K20" s="89">
         <f>IF($N11=0,0,$P11*K11/$N11)</f>
-        <v/>
+        <v>28.3414059444846</v>
       </c>
       <c r="L20" s="89">
         <f>IF($N11=0,0,$P11*L11/$N11)</f>
-        <v/>
+        <v>36.0708802929802</v>
       </c>
       <c r="M20" s="89">
         <f>IF($N11=0,0,$P11*M11/$N11)</f>
-        <v/>
+        <v>43.8003546414761</v>
       </c>
       <c r="N20" s="89">
         <f>SUM(B20:M20)</f>
-        <v/>
+        <v>257.649144949859</v>
       </c>
       <c r="O20" s="89" t="n"/>
       <c r="P20" s="89" t="n"/>
@@ -3292,55 +3303,55 @@
       </c>
       <c r="B21" s="92">
         <f>B15</f>
-        <v/>
+        <v>30.0166839504208</v>
       </c>
       <c r="C21" s="92">
         <f>C15</f>
-        <v/>
+        <v>75.0417098760519</v>
       </c>
       <c r="D21" s="92">
         <f>D15</f>
-        <v/>
+        <v>105.058393826473</v>
       </c>
       <c r="E21" s="92">
         <f>E15</f>
-        <v/>
+        <v>105.058393826472</v>
       </c>
       <c r="F21" s="92">
         <f>F15</f>
-        <v/>
+        <v>105.058393826473</v>
       </c>
       <c r="G21" s="92">
         <f>G15</f>
-        <v/>
+        <v>105.058393826473</v>
       </c>
       <c r="H21" s="92">
         <f>H15</f>
-        <v/>
+        <v>105.058393826473</v>
       </c>
       <c r="I21" s="92">
         <f>I15</f>
-        <v/>
+        <v>120.066735801683</v>
       </c>
       <c r="J21" s="92">
         <f>J15</f>
-        <v/>
+        <v>120.066735801683</v>
       </c>
       <c r="K21" s="92">
         <f>K15</f>
-        <v/>
+        <v>165.091761727314</v>
       </c>
       <c r="L21" s="92">
         <f>L15</f>
-        <v/>
+        <v>210.116787652944</v>
       </c>
       <c r="M21" s="92">
         <f>M15</f>
-        <v/>
+        <v>255.141813578577</v>
       </c>
       <c r="N21" s="92">
         <f>N15</f>
-        <v/>
+        <v>1500.83419752104</v>
       </c>
       <c r="O21" s="89" t="n"/>
       <c r="P21" s="89" t="n"/>
@@ -3353,55 +3364,55 @@
       </c>
       <c r="B22" s="92">
         <f>B16+B17+B18+B19+B20</f>
-        <v/>
+        <v>54.8394530098368</v>
       </c>
       <c r="C22" s="92">
         <f>C16+C17+C18+C19+C20</f>
-        <v/>
+        <v>137.100380772931</v>
       </c>
       <c r="D22" s="92">
         <f>D16+D17+D18+D19+D20</f>
-        <v/>
+        <v>191.938085534429</v>
       </c>
       <c r="E22" s="92">
         <f>E16+E17+E18+E19+E20</f>
-        <v/>
+        <v>191.93284078941</v>
       </c>
       <c r="F22" s="92">
         <f>F16+F17+F18+F19+F20</f>
-        <v/>
+        <v>191.938085534429</v>
       </c>
       <c r="G22" s="92">
         <f>G16+G17+G18+G19+G20</f>
-        <v/>
+        <v>191.938085534429</v>
       </c>
       <c r="H22" s="92">
         <f>H16+H17+H18+H19+H20</f>
-        <v/>
+        <v>191.938085534429</v>
       </c>
       <c r="I22" s="92">
         <f>I16+I17+I18+I19+I20</f>
-        <v/>
+        <v>219.34907079765</v>
       </c>
       <c r="J22" s="92">
         <f>J16+J17+J18+J19+J20</f>
-        <v/>
+        <v>219.34907079765</v>
       </c>
       <c r="K22" s="92">
         <f>K16+K17+K18+K19+K20</f>
-        <v/>
+        <v>301.616991554103</v>
       </c>
       <c r="L22" s="92">
         <f>L16+L17+L18+L19+L20</f>
-        <v/>
+        <v>383.876171068858</v>
       </c>
       <c r="M22" s="92">
         <f>M16+M17+M18+M19+M20</f>
-        <v/>
+        <v>466.135350583613</v>
       </c>
       <c r="N22" s="92">
         <f>N16+N17+N18+N19+N20</f>
-        <v/>
+        <v>2741.95167151177</v>
       </c>
       <c r="O22" s="89" t="n"/>
       <c r="P22" s="89" t="n"/>
@@ -3414,55 +3425,55 @@
       </c>
       <c r="B23" s="90">
         <f>B21+B22</f>
-        <v/>
+        <v>84.8561369602576</v>
       </c>
       <c r="C23" s="90">
         <f>C21+C22</f>
-        <v/>
+        <v>212.142090648983</v>
       </c>
       <c r="D23" s="90">
         <f>D21+D22</f>
-        <v/>
+        <v>296.996479360902</v>
       </c>
       <c r="E23" s="90">
         <f>E21+E22</f>
-        <v/>
+        <v>296.991234615883</v>
       </c>
       <c r="F23" s="90">
         <f>F21+F22</f>
-        <v/>
+        <v>296.996479360902</v>
       </c>
       <c r="G23" s="90">
         <f>G21+G22</f>
-        <v/>
+        <v>296.996479360902</v>
       </c>
       <c r="H23" s="90">
         <f>H21+H22</f>
-        <v/>
+        <v>296.996479360902</v>
       </c>
       <c r="I23" s="90">
         <f>I21+I22</f>
-        <v/>
+        <v>339.415806599333</v>
       </c>
       <c r="J23" s="90">
         <f>J21+J22</f>
-        <v/>
+        <v>339.415806599333</v>
       </c>
       <c r="K23" s="90">
         <f>K21+K22</f>
-        <v/>
+        <v>466.708753281417</v>
       </c>
       <c r="L23" s="90">
         <f>L21+L22</f>
-        <v/>
+        <v>593.992958721802</v>
       </c>
       <c r="M23" s="90">
         <f>M21+M22</f>
-        <v/>
+        <v>721.27716416219</v>
       </c>
       <c r="N23" s="90">
         <f>N21+N22</f>
-        <v/>
+        <v>4242.78586903281</v>
       </c>
       <c r="O23" s="89" t="n"/>
       <c r="P23" s="89" t="n"/>
@@ -3550,7 +3561,7 @@
       </c>
       <c r="N26" s="89">
         <f>SUM(B26:M26)</f>
-        <v/>
+        <v>-1000</v>
       </c>
       <c r="O26" s="89" t="n"/>
       <c r="P26" s="89" t="n"/>
@@ -3599,7 +3610,7 @@
       </c>
       <c r="N27" s="89">
         <f>SUM(B27:M27)</f>
-        <v/>
+        <v>-795</v>
       </c>
       <c r="O27" s="89" t="n"/>
       <c r="P27" s="89" t="n"/>
@@ -3648,7 +3659,7 @@
       </c>
       <c r="N28" s="89">
         <f>SUM(B28:M28)</f>
-        <v/>
+        <v>-176.066</v>
       </c>
       <c r="O28" s="89" t="n"/>
       <c r="P28" s="89" t="n"/>
@@ -3661,55 +3672,55 @@
       </c>
       <c r="B29" s="90">
         <f>B26+B27+B28</f>
-        <v/>
+        <v>-89.8692999412308</v>
       </c>
       <c r="C29" s="90">
         <f>C26+C27+C28</f>
-        <v/>
+        <v>-125.27429364453</v>
       </c>
       <c r="D29" s="90">
         <f>D26+D27+D28</f>
-        <v/>
+        <v>-148.837732616909</v>
       </c>
       <c r="E29" s="90">
         <f>E26+E27+E28</f>
-        <v/>
+        <v>-152.621631349173</v>
       </c>
       <c r="F29" s="90">
         <f>F26+F27+F28</f>
-        <v/>
+        <v>-153.651031416338</v>
       </c>
       <c r="G29" s="90">
         <f>G26+G27+G28</f>
-        <v/>
+        <v>-154.559410796743</v>
       </c>
       <c r="H29" s="90">
         <f>H26+H27+H28</f>
-        <v/>
+        <v>-154.512725178407</v>
       </c>
       <c r="I29" s="90">
         <f>I26+I27+I28</f>
-        <v/>
+        <v>-164.495994710772</v>
       </c>
       <c r="J29" s="90">
         <f>J26+J27+J28</f>
-        <v/>
+        <v>-161.961631987239</v>
       </c>
       <c r="K29" s="90">
         <f>K26+K27+K28</f>
-        <v/>
+        <v>-197.159261674083</v>
       </c>
       <c r="L29" s="90">
         <f>L26+L27+L28</f>
-        <v/>
+        <v>-218.989611938544</v>
       </c>
       <c r="M29" s="90">
         <f>M26+M27+M28</f>
-        <v/>
+        <v>-249.133374746033</v>
       </c>
       <c r="N29" s="90">
         <f>N26+N27+N28</f>
-        <v/>
+        <v>-1971.066</v>
       </c>
       <c r="O29" s="89" t="n"/>
       <c r="P29" s="89" t="n"/>
@@ -3758,7 +3769,7 @@
       </c>
       <c r="N30" s="89">
         <f>SUM(B30:M30)</f>
-        <v/>
+        <v>-1436.36293659997</v>
       </c>
       <c r="O30" s="89" t="n"/>
       <c r="P30" s="89" t="n"/>
@@ -3807,7 +3818,7 @@
       </c>
       <c r="N31" s="89">
         <f>SUM(B31:M31)</f>
-        <v/>
+        <v>-40.2864319085485</v>
       </c>
       <c r="O31" s="89" t="n"/>
       <c r="P31" s="89" t="n"/>
@@ -3856,7 +3867,7 @@
       </c>
       <c r="N32" s="89">
         <f>SUM(B32:M32)</f>
-        <v/>
+        <v>-2071.724216</v>
       </c>
       <c r="O32" s="89" t="n"/>
       <c r="P32" s="89" t="n"/>
@@ -3869,55 +3880,55 @@
       </c>
       <c r="B33" s="89">
         <f>B32-B29</f>
-        <v/>
+        <v>-5.9676922666667</v>
       </c>
       <c r="C33" s="89">
         <f>C32-C29</f>
-        <v/>
+        <v>-10.3176922666667</v>
       </c>
       <c r="D33" s="89">
         <f>D32-D29</f>
-        <v/>
+        <v>-9.54269226666631</v>
       </c>
       <c r="E33" s="89">
         <f>E32-E29</f>
-        <v/>
+        <v>-7.967692266667</v>
       </c>
       <c r="F33" s="89">
         <f>F32-F29</f>
-        <v/>
+        <v>-6.16769226666722</v>
       </c>
       <c r="G33" s="89">
         <f>G32-G29</f>
-        <v/>
+        <v>-7.34269226666646</v>
       </c>
       <c r="H33" s="89">
         <f>H32-H29</f>
-        <v/>
+        <v>-10.3086770666665</v>
       </c>
       <c r="I33" s="89">
         <f>I32-I29</f>
-        <v/>
+        <v>-7.6586770666664</v>
       </c>
       <c r="J33" s="89">
         <f>J32-J29</f>
-        <v/>
+        <v>-9.2336770666663</v>
       </c>
       <c r="K33" s="89">
         <f>K32-K29</f>
-        <v/>
+        <v>-7.60867706666699</v>
       </c>
       <c r="L33" s="89">
         <f>L32-L29</f>
-        <v/>
+        <v>-11.508677066667</v>
       </c>
       <c r="M33" s="89">
         <f>M32-M29</f>
-        <v/>
+        <v>-7.033677066667</v>
       </c>
       <c r="N33" s="89">
         <f>N32-N29</f>
-        <v/>
+        <v>-100.658216000001</v>
       </c>
       <c r="O33" s="89" t="n"/>
       <c r="P33" s="89" t="n"/>
@@ -3966,7 +3977,7 @@
       </c>
       <c r="N34" s="89">
         <f>SUM(B34:M34)</f>
-        <v/>
+        <v>-92.1005567838379</v>
       </c>
       <c r="O34" s="89" t="n"/>
       <c r="P34" s="89" t="n"/>
@@ -4015,7 +4026,7 @@
       </c>
       <c r="N35" s="89">
         <f>SUM(B35:M35)</f>
-        <v/>
+        <v>-102.312181722681</v>
       </c>
       <c r="O35" s="89" t="n"/>
       <c r="P35" s="89" t="n"/>
@@ -4067,55 +4078,55 @@
       </c>
       <c r="B38" s="90">
         <f>B23+B29</f>
-        <v/>
+        <v>-5.01316298097319</v>
       </c>
       <c r="C38" s="90">
         <f>C23+C29</f>
-        <v/>
+        <v>86.8677970044529</v>
       </c>
       <c r="D38" s="90">
         <f>D23+D29</f>
-        <v/>
+        <v>148.158746743993</v>
       </c>
       <c r="E38" s="90">
         <f>E23+E29</f>
-        <v/>
+        <v>144.36960326671</v>
       </c>
       <c r="F38" s="90">
         <f>F23+F29</f>
-        <v/>
+        <v>143.345447944564</v>
       </c>
       <c r="G38" s="90">
         <f>G23+G29</f>
-        <v/>
+        <v>142.437068564159</v>
       </c>
       <c r="H38" s="90">
         <f>H23+H29</f>
-        <v/>
+        <v>142.483754182495</v>
       </c>
       <c r="I38" s="90">
         <f>I23+I29</f>
-        <v/>
+        <v>174.919811888561</v>
       </c>
       <c r="J38" s="90">
         <f>J23+J29</f>
-        <v/>
+        <v>177.454174612094</v>
       </c>
       <c r="K38" s="90">
         <f>K23+K29</f>
-        <v/>
+        <v>269.549491607334</v>
       </c>
       <c r="L38" s="90">
         <f>L23+L29</f>
-        <v/>
+        <v>375.003346783258</v>
       </c>
       <c r="M38" s="90">
         <f>M23+M29</f>
-        <v/>
+        <v>472.143789416157</v>
       </c>
       <c r="N38" s="90">
         <f>N23+N29</f>
-        <v/>
+        <v>2271.71986903281</v>
       </c>
       <c r="O38" s="89" t="n"/>
       <c r="P38" s="89" t="n"/>
@@ -4128,55 +4139,55 @@
       </c>
       <c r="B39" s="92">
         <f>B30+B31</f>
-        <v/>
+        <v>-115.120241402344</v>
       </c>
       <c r="C39" s="92">
         <f>C30+C31</f>
-        <v/>
+        <v>-121.257358977713</v>
       </c>
       <c r="D39" s="92">
         <f>D30+D31</f>
-        <v/>
+        <v>-118.513853826792</v>
       </c>
       <c r="E39" s="92">
         <f>E30+E31</f>
-        <v/>
+        <v>-130.916128192984</v>
       </c>
       <c r="F39" s="92">
         <f>F30+F31</f>
-        <v/>
+        <v>-122.546333750311</v>
       </c>
       <c r="G39" s="92">
         <f>G30+G31</f>
-        <v/>
+        <v>-119.501886301288</v>
       </c>
       <c r="H39" s="92">
         <f>H30+H31</f>
-        <v/>
+        <v>-128.587363594834</v>
       </c>
       <c r="I39" s="92">
         <f>I30+I31</f>
-        <v/>
+        <v>-104.886573994631</v>
       </c>
       <c r="J39" s="92">
         <f>J30+J31</f>
-        <v/>
+        <v>-121.513263931605</v>
       </c>
       <c r="K39" s="92">
         <f>K30+K31</f>
-        <v/>
+        <v>-129.632256627366</v>
       </c>
       <c r="L39" s="92">
         <f>L30+L31</f>
-        <v/>
+        <v>-129.699373530037</v>
       </c>
       <c r="M39" s="92">
         <f>M30+M31</f>
-        <v/>
+        <v>-134.474734378612</v>
       </c>
       <c r="N39" s="92">
         <f>N30+N31</f>
-        <v/>
+        <v>-1476.64936850852</v>
       </c>
       <c r="O39" s="89" t="n"/>
       <c r="P39" s="89" t="n"/>
@@ -4189,55 +4200,55 @@
       </c>
       <c r="B40" s="92">
         <f>B33+B34+B35</f>
-        <v/>
+        <v>-14.8620161334858</v>
       </c>
       <c r="C40" s="92">
         <f>C33+C34+C35</f>
-        <v/>
+        <v>-22.0924241030238</v>
       </c>
       <c r="D40" s="92">
         <f>D33+D34+D35</f>
-        <v/>
+        <v>-23.6376439774978</v>
       </c>
       <c r="E40" s="92">
         <f>E33+E34+E35</f>
-        <v/>
+        <v>-21.8625501881068</v>
       </c>
       <c r="F40" s="92">
         <f>F33+F34+F35</f>
-        <v/>
+        <v>-20.5626439774987</v>
       </c>
       <c r="G40" s="92">
         <f>G33+G34+G35</f>
-        <v/>
+        <v>-21.6881509284325</v>
       </c>
       <c r="H40" s="92">
         <f>H33+H34+H35</f>
-        <v/>
+        <v>-24.5965628215011</v>
       </c>
       <c r="I40" s="92">
         <f>I33+I34+I35</f>
-        <v/>
+        <v>-23.1744683152784</v>
       </c>
       <c r="J40" s="92">
         <f>J33+J34+J35</f>
-        <v/>
+        <v>-26.2608668883188</v>
       </c>
       <c r="K40" s="92">
         <f>K33+K34+K35</f>
-        <v/>
+        <v>-28.122499018051</v>
       </c>
       <c r="L40" s="92">
         <f>L33+L34+L35</f>
-        <v/>
+        <v>-34.9028757244585</v>
       </c>
       <c r="M40" s="92">
         <f>M33+M34+M35</f>
-        <v/>
+        <v>-33.3082524308659</v>
       </c>
       <c r="N40" s="92">
         <f>N33+N34+N35</f>
-        <v/>
+        <v>-295.070954506519</v>
       </c>
       <c r="O40" s="89" t="n"/>
       <c r="P40" s="89" t="n"/>
@@ -4250,55 +4261,55 @@
       </c>
       <c r="B41" s="90">
         <f>B39+B40</f>
-        <v/>
+        <v>-129.98225753583</v>
       </c>
       <c r="C41" s="90">
         <f>C39+C40</f>
-        <v/>
+        <v>-143.349783080737</v>
       </c>
       <c r="D41" s="90">
         <f>D39+D40</f>
-        <v/>
+        <v>-142.15149780429</v>
       </c>
       <c r="E41" s="90">
         <f>E39+E40</f>
-        <v/>
+        <v>-152.778678381091</v>
       </c>
       <c r="F41" s="90">
         <f>F39+F40</f>
-        <v/>
+        <v>-143.10897772781</v>
       </c>
       <c r="G41" s="90">
         <f>G39+G40</f>
-        <v/>
+        <v>-141.190037229721</v>
       </c>
       <c r="H41" s="90">
         <f>H39+H40</f>
-        <v/>
+        <v>-153.183926416335</v>
       </c>
       <c r="I41" s="90">
         <f>I39+I40</f>
-        <v/>
+        <v>-128.06104230991</v>
       </c>
       <c r="J41" s="90">
         <f>J39+J40</f>
-        <v/>
+        <v>-147.774130819924</v>
       </c>
       <c r="K41" s="90">
         <f>K39+K40</f>
-        <v/>
+        <v>-157.754755645417</v>
       </c>
       <c r="L41" s="90">
         <f>L39+L40</f>
-        <v/>
+        <v>-164.602249254496</v>
       </c>
       <c r="M41" s="90">
         <f>M39+M40</f>
-        <v/>
+        <v>-167.782986809477</v>
       </c>
       <c r="N41" s="90">
         <f>N39+N40</f>
-        <v/>
+        <v>-1771.72032301504</v>
       </c>
       <c r="O41" s="89" t="n"/>
       <c r="P41" s="89" t="n"/>
@@ -4311,55 +4322,55 @@
       </c>
       <c r="B42" s="90">
         <f>B38+B41</f>
-        <v/>
+        <v>-134.995420516803</v>
       </c>
       <c r="C42" s="90">
         <f>C38+C41</f>
-        <v/>
+        <v>-56.481986076284</v>
       </c>
       <c r="D42" s="90">
         <f>D38+D41</f>
-        <v/>
+        <v>6.00724893970295</v>
       </c>
       <c r="E42" s="90">
         <f>E38+E41</f>
-        <v/>
+        <v>-8.40907511438118</v>
       </c>
       <c r="F42" s="90">
         <f>F38+F41</f>
-        <v/>
+        <v>0.236470216753929</v>
       </c>
       <c r="G42" s="90">
         <f>G38+G41</f>
-        <v/>
+        <v>1.24703133443836</v>
       </c>
       <c r="H42" s="90">
         <f>H38+H41</f>
-        <v/>
+        <v>-10.7001722338402</v>
       </c>
       <c r="I42" s="90">
         <f>I38+I41</f>
-        <v/>
+        <v>46.8587695786517</v>
       </c>
       <c r="J42" s="90">
         <f>J38+J41</f>
-        <v/>
+        <v>29.6800437921701</v>
       </c>
       <c r="K42" s="90">
         <f>K38+K41</f>
-        <v/>
+        <v>111.794735961916</v>
       </c>
       <c r="L42" s="90">
         <f>L38+L41</f>
-        <v/>
+        <v>210.401097528762</v>
       </c>
       <c r="M42" s="90">
         <f>M38+M41</f>
-        <v/>
+        <v>304.36080260668</v>
       </c>
       <c r="N42" s="90">
         <f>N38+N41</f>
-        <v/>
+        <v>499.999546017767</v>
       </c>
       <c r="O42" s="89" t="n"/>
       <c r="P42" s="89" t="n"/>
@@ -4401,7 +4412,7 @@
       <c r="M44" s="89" t="n"/>
       <c r="N44" s="89">
         <f>ROUND(N42-499.999546017767,3)</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="O44" s="89" t="n"/>
       <c r="P44" s="89" t="n"/>
@@ -4411,4 +4422,2933 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A2:N4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="51.83" customWidth="1" style="48" min="1" max="1"/>
+    <col width="14.16" customWidth="1" style="48" min="2" max="2"/>
+    <col width="14.16" customWidth="1" style="48" min="3" max="3"/>
+    <col width="14.16" customWidth="1" style="48" min="4" max="4"/>
+    <col width="14.16" customWidth="1" style="48" min="5" max="5"/>
+    <col width="14.16" customWidth="1" style="48" min="6" max="6"/>
+    <col width="14.16" customWidth="1" style="48" min="7" max="7"/>
+    <col width="14.16" customWidth="1" style="48" min="8" max="8"/>
+    <col width="14.16" customWidth="1" style="48" min="9" max="9"/>
+    <col width="14.16" customWidth="1" style="48" min="10" max="10"/>
+    <col width="14.16" customWidth="1" style="48" min="11" max="11"/>
+    <col width="14.16" customWidth="1" style="48" min="12" max="12"/>
+    <col width="14.16" customWidth="1" style="48" min="13" max="13"/>
+    <col width="14.16" customWidth="1" style="48" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="15.75" customHeight="1" s="48">
+      <c r="B2" s="49" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="C2" s="49" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="D2" s="49" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="E2" s="49" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="F2" s="49" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="G2" s="49" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="H2" s="49" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="I2" s="49" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="J2" s="49" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="K2" s="50" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="L2" s="50" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+      <c r="M2" s="50" t="inlineStr">
+        <is>
+          <t>бюджет</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1" s="48">
+      <c r="A3" s="52" t="inlineStr">
+        <is>
+          <t>CAPEX, RUB</t>
+        </is>
+      </c>
+      <c r="B3" s="53" t="inlineStr">
+        <is>
+          <t>jan'27</t>
+        </is>
+      </c>
+      <c r="C3" s="53" t="inlineStr">
+        <is>
+          <t>feb'27</t>
+        </is>
+      </c>
+      <c r="D3" s="53" t="inlineStr">
+        <is>
+          <t>mar'27</t>
+        </is>
+      </c>
+      <c r="E3" s="53" t="inlineStr">
+        <is>
+          <t>apr'27</t>
+        </is>
+      </c>
+      <c r="F3" s="53" t="inlineStr">
+        <is>
+          <t>may'27</t>
+        </is>
+      </c>
+      <c r="G3" s="53" t="inlineStr">
+        <is>
+          <t>jun'27</t>
+        </is>
+      </c>
+      <c r="H3" s="53" t="inlineStr">
+        <is>
+          <t>jul'27</t>
+        </is>
+      </c>
+      <c r="I3" s="53" t="inlineStr">
+        <is>
+          <t>aug'27</t>
+        </is>
+      </c>
+      <c r="J3" s="53" t="inlineStr">
+        <is>
+          <t>sep'27</t>
+        </is>
+      </c>
+      <c r="K3" s="53" t="inlineStr">
+        <is>
+          <t>oct'27</t>
+        </is>
+      </c>
+      <c r="L3" s="53" t="inlineStr">
+        <is>
+          <t>nov'27</t>
+        </is>
+      </c>
+      <c r="M3" s="53" t="inlineStr">
+        <is>
+          <t>dec'27</t>
+        </is>
+      </c>
+      <c r="N3" s="53" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="15" customHeight="1" s="48">
+      <c r="A4" s="69" t="inlineStr">
+        <is>
+          <t>CAPEX</t>
+        </is>
+      </c>
+      <c r="B4" s="70" t="n">
+        <v>-42458922.15706224</v>
+      </c>
+      <c r="C4" s="70" t="n">
+        <v>-43045580.11446574</v>
+      </c>
+      <c r="D4" s="70" t="n">
+        <v>-44505900.84302051</v>
+      </c>
+      <c r="E4" s="70" t="n">
+        <v>-54600359.20961371</v>
+      </c>
+      <c r="F4" s="70" t="n">
+        <v>-62889771.82107642</v>
+      </c>
+      <c r="G4" s="70" t="n">
+        <v>-96755462.89143273</v>
+      </c>
+      <c r="H4" s="70" t="n">
+        <v>-92787182.57526618</v>
+      </c>
+      <c r="I4" s="70" t="n">
+        <v>-103242998.3992597</v>
+      </c>
+      <c r="J4" s="70" t="n">
+        <v>-201652626.2744877</v>
+      </c>
+      <c r="K4" s="70" t="n">
+        <v>-216825839.570551</v>
+      </c>
+      <c r="L4" s="70" t="n">
+        <v>-45970661.13664418</v>
+      </c>
+      <c r="M4" s="70" t="n">
+        <v>-145904436.886102</v>
+      </c>
+      <c r="N4" s="70">
+        <f>SUM(B4:M4)</f>
+        <v>-1150639741.87898</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr filterMode="0">
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="0"/>
+  </sheetPr>
+  <dimension ref="A2:N64"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="8.83203125" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
+  <cols>
+    <col width="51.83" customWidth="1" style="46" min="1" max="1"/>
+    <col width="14.16" customWidth="1" style="46" min="2" max="13"/>
+    <col width="11.16" customWidth="1" style="47" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="15.75" customHeight="1" s="48">
+      <c r="B2" s="49" t="inlineStr">
+        <is>
+          <t>факт</t>
+        </is>
+      </c>
+      <c r="C2" s="49" t="inlineStr">
+        <is>
+          <t>факт</t>
+        </is>
+      </c>
+      <c r="D2" s="49" t="inlineStr">
+        <is>
+          <t>факт</t>
+        </is>
+      </c>
+      <c r="E2" s="49" t="inlineStr">
+        <is>
+          <t>факт</t>
+        </is>
+      </c>
+      <c r="F2" s="49" t="inlineStr">
+        <is>
+          <t>факт</t>
+        </is>
+      </c>
+      <c r="G2" s="49" t="inlineStr">
+        <is>
+          <t>факт</t>
+        </is>
+      </c>
+      <c r="H2" s="49" t="inlineStr">
+        <is>
+          <t>факт</t>
+        </is>
+      </c>
+      <c r="I2" s="49" t="inlineStr">
+        <is>
+          <t>факт</t>
+        </is>
+      </c>
+      <c r="J2" s="49" t="inlineStr">
+        <is>
+          <t>факт</t>
+        </is>
+      </c>
+      <c r="K2" s="93" t="inlineStr">
+        <is>
+          <t>прогноз</t>
+        </is>
+      </c>
+      <c r="L2" s="93" t="inlineStr">
+        <is>
+          <t>прогноз</t>
+        </is>
+      </c>
+      <c r="M2" s="93" t="inlineStr">
+        <is>
+          <t>прогноз</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A3" s="52" t="inlineStr">
+        <is>
+          <t>P&amp;L, RUB</t>
+        </is>
+      </c>
+      <c r="B3" s="53" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C3" s="53" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D3" s="53" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E3" s="53" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F3" s="53" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G3" s="53" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H3" s="53" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I3" s="53" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J3" s="53" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K3" s="53" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L3" s="53" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M3" s="53" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N3" s="54" t="n"/>
+    </row>
+    <row r="4" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A4" s="55" t="inlineStr">
+        <is>
+          <t>Orders</t>
+        </is>
+      </c>
+      <c r="B4" s="56" t="n"/>
+      <c r="C4" s="56" t="n"/>
+      <c r="D4" s="56" t="n"/>
+      <c r="E4" s="56" t="n"/>
+      <c r="F4" s="56" t="n"/>
+      <c r="G4" s="56" t="n"/>
+      <c r="H4" s="56" t="n"/>
+      <c r="I4" s="56" t="n"/>
+      <c r="J4" s="56" t="n"/>
+      <c r="K4" s="56" t="n"/>
+      <c r="L4" s="56" t="n"/>
+      <c r="M4" s="56" t="n"/>
+      <c r="N4" s="54" t="n"/>
+    </row>
+    <row r="5" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A5" s="57" t="inlineStr">
+        <is>
+          <t>Own service</t>
+        </is>
+      </c>
+      <c r="B5" s="58" t="n"/>
+      <c r="C5" s="58" t="n"/>
+      <c r="D5" s="58" t="n"/>
+      <c r="E5" s="58" t="n"/>
+      <c r="F5" s="58" t="n"/>
+      <c r="G5" s="58" t="n"/>
+      <c r="H5" s="58" t="n"/>
+      <c r="I5" s="58" t="n"/>
+      <c r="J5" s="58" t="n"/>
+      <c r="K5" s="58" t="n"/>
+      <c r="L5" s="58" t="n"/>
+      <c r="M5" s="58" t="n"/>
+      <c r="N5" s="54" t="n"/>
+    </row>
+    <row r="6" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A6" s="57" t="inlineStr">
+        <is>
+          <t>Partners service</t>
+        </is>
+      </c>
+      <c r="B6" s="59" t="n"/>
+      <c r="C6" s="59" t="n"/>
+      <c r="D6" s="59" t="n"/>
+      <c r="E6" s="59" t="n"/>
+      <c r="F6" s="59" t="n"/>
+      <c r="G6" s="59" t="n"/>
+      <c r="H6" s="59" t="n"/>
+      <c r="I6" s="59" t="n"/>
+      <c r="J6" s="59" t="n"/>
+      <c r="K6" s="59" t="n"/>
+      <c r="L6" s="59" t="n"/>
+      <c r="M6" s="59" t="n"/>
+      <c r="N6" s="54" t="n"/>
+    </row>
+    <row r="7" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A7" s="55" t="inlineStr">
+        <is>
+          <t>Gross Revenue</t>
+        </is>
+      </c>
+      <c r="B7" s="56" t="n"/>
+      <c r="C7" s="56" t="n"/>
+      <c r="D7" s="56" t="n"/>
+      <c r="E7" s="56" t="n"/>
+      <c r="F7" s="56" t="n"/>
+      <c r="G7" s="56" t="n"/>
+      <c r="H7" s="56" t="n"/>
+      <c r="I7" s="56" t="n"/>
+      <c r="J7" s="56" t="n"/>
+      <c r="K7" s="56" t="n"/>
+      <c r="L7" s="56" t="n"/>
+      <c r="M7" s="56" t="n"/>
+      <c r="N7" s="54" t="n"/>
+    </row>
+    <row r="8" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A8" s="57" t="inlineStr">
+        <is>
+          <t>Own service</t>
+        </is>
+      </c>
+      <c r="B8" s="56" t="n"/>
+      <c r="C8" s="56" t="n"/>
+      <c r="D8" s="56" t="n"/>
+      <c r="E8" s="56" t="n"/>
+      <c r="F8" s="56" t="n"/>
+      <c r="G8" s="56" t="n"/>
+      <c r="H8" s="56" t="n"/>
+      <c r="I8" s="56" t="n"/>
+      <c r="J8" s="56" t="n"/>
+      <c r="K8" s="56" t="n"/>
+      <c r="L8" s="56" t="n"/>
+      <c r="M8" s="56" t="n"/>
+      <c r="N8" s="54" t="n"/>
+    </row>
+    <row r="9" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A9" s="57" t="inlineStr">
+        <is>
+          <t>Partners service</t>
+        </is>
+      </c>
+      <c r="B9" s="60" t="n"/>
+      <c r="C9" s="60" t="n"/>
+      <c r="D9" s="60" t="n"/>
+      <c r="E9" s="60" t="n"/>
+      <c r="F9" s="60" t="n"/>
+      <c r="G9" s="60" t="n"/>
+      <c r="H9" s="60" t="n"/>
+      <c r="I9" s="60" t="n"/>
+      <c r="J9" s="60" t="n"/>
+      <c r="K9" s="60" t="n"/>
+      <c r="L9" s="60" t="n"/>
+      <c r="M9" s="60" t="n"/>
+      <c r="N9" s="54" t="n"/>
+    </row>
+    <row r="10" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A10" s="55" t="inlineStr">
+        <is>
+          <t>Promo incl Loyalty</t>
+        </is>
+      </c>
+      <c r="B10" s="56" t="n"/>
+      <c r="C10" s="56" t="n"/>
+      <c r="D10" s="56" t="n"/>
+      <c r="E10" s="56" t="n"/>
+      <c r="F10" s="56" t="n"/>
+      <c r="G10" s="56" t="n"/>
+      <c r="H10" s="56" t="n"/>
+      <c r="I10" s="56" t="n"/>
+      <c r="J10" s="56" t="n"/>
+      <c r="K10" s="56" t="n"/>
+      <c r="L10" s="56" t="n"/>
+      <c r="M10" s="56" t="n"/>
+      <c r="N10" s="54" t="n"/>
+    </row>
+    <row r="11" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A11" s="57" t="inlineStr">
+        <is>
+          <t>Own service</t>
+        </is>
+      </c>
+      <c r="B11" s="56" t="n"/>
+      <c r="C11" s="56" t="n"/>
+      <c r="D11" s="56" t="n"/>
+      <c r="E11" s="56" t="n"/>
+      <c r="F11" s="56" t="n"/>
+      <c r="G11" s="56" t="n"/>
+      <c r="H11" s="56" t="n"/>
+      <c r="I11" s="56" t="n"/>
+      <c r="J11" s="56" t="n"/>
+      <c r="K11" s="56" t="n"/>
+      <c r="L11" s="56" t="n"/>
+      <c r="M11" s="56" t="n"/>
+      <c r="N11" s="54" t="n"/>
+    </row>
+    <row r="12" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A12" s="57" t="inlineStr">
+        <is>
+          <t>Partners service</t>
+        </is>
+      </c>
+      <c r="B12" s="61" t="n"/>
+      <c r="C12" s="61" t="n"/>
+      <c r="D12" s="61" t="n"/>
+      <c r="E12" s="61" t="n"/>
+      <c r="F12" s="61" t="n"/>
+      <c r="G12" s="61" t="n"/>
+      <c r="H12" s="61" t="n"/>
+      <c r="I12" s="61" t="n"/>
+      <c r="J12" s="61" t="n"/>
+      <c r="K12" s="61" t="n"/>
+      <c r="L12" s="61" t="n"/>
+      <c r="M12" s="61" t="n"/>
+      <c r="N12" s="54" t="n"/>
+    </row>
+    <row r="13" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A13" s="55" t="inlineStr">
+        <is>
+          <t>Net Revenue</t>
+        </is>
+      </c>
+      <c r="B13" s="56" t="n"/>
+      <c r="C13" s="56" t="n"/>
+      <c r="D13" s="56" t="n"/>
+      <c r="E13" s="56" t="n"/>
+      <c r="F13" s="56" t="n"/>
+      <c r="G13" s="56" t="n"/>
+      <c r="H13" s="56" t="n"/>
+      <c r="I13" s="56" t="n"/>
+      <c r="J13" s="56" t="n"/>
+      <c r="K13" s="56" t="n"/>
+      <c r="L13" s="56" t="n"/>
+      <c r="M13" s="56" t="n"/>
+      <c r="N13" s="54" t="n"/>
+    </row>
+    <row r="14" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A14" s="57" t="inlineStr">
+        <is>
+          <t>Own service</t>
+        </is>
+      </c>
+      <c r="B14" s="56" t="n"/>
+      <c r="C14" s="56" t="n"/>
+      <c r="D14" s="56" t="n"/>
+      <c r="E14" s="56" t="n"/>
+      <c r="F14" s="56" t="n"/>
+      <c r="G14" s="56" t="n"/>
+      <c r="H14" s="56" t="n"/>
+      <c r="I14" s="56" t="n"/>
+      <c r="J14" s="56" t="n"/>
+      <c r="K14" s="56" t="n"/>
+      <c r="L14" s="56" t="n"/>
+      <c r="M14" s="56" t="n"/>
+      <c r="N14" s="54" t="n"/>
+    </row>
+    <row r="15" hidden="1" ht="14.25" customFormat="1" customHeight="1" s="51">
+      <c r="A15" s="57" t="inlineStr">
+        <is>
+          <t>Partners service</t>
+        </is>
+      </c>
+      <c r="B15" s="61" t="n"/>
+      <c r="C15" s="61" t="n"/>
+      <c r="D15" s="61" t="n"/>
+      <c r="E15" s="61" t="n"/>
+      <c r="F15" s="61" t="n"/>
+      <c r="G15" s="61" t="n"/>
+      <c r="H15" s="61" t="n"/>
+      <c r="I15" s="61" t="n"/>
+      <c r="J15" s="61" t="n"/>
+      <c r="K15" s="61" t="n"/>
+      <c r="L15" s="61" t="n"/>
+      <c r="M15" s="61" t="n"/>
+      <c r="N15" s="54" t="n"/>
+    </row>
+    <row r="16" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A16" s="55" t="inlineStr">
+        <is>
+          <t>Commercial margin</t>
+        </is>
+      </c>
+      <c r="B16" s="56" t="n">
+        <v>51397105.34437963</v>
+      </c>
+      <c r="C16" s="56" t="n">
+        <v>139325480.6976929</v>
+      </c>
+      <c r="D16" s="56" t="n">
+        <v>142508217.7192157</v>
+      </c>
+      <c r="E16" s="56" t="n">
+        <v>74530640.26743269</v>
+      </c>
+      <c r="F16" s="56" t="n">
+        <v>290925019.5202637</v>
+      </c>
+      <c r="G16" s="56" t="n">
+        <v>342575263.6328037</v>
+      </c>
+      <c r="H16" s="56" t="n">
+        <v>143329946.9682095</v>
+      </c>
+      <c r="I16" s="56" t="n">
+        <v>177328700.0704224</v>
+      </c>
+      <c r="J16" s="56" t="n">
+        <v>335398417.4200364</v>
+      </c>
+      <c r="K16" s="56" t="n">
+        <v>87471840.42115504</v>
+      </c>
+      <c r="L16" s="56" t="n">
+        <v>211633363.2039606</v>
+      </c>
+      <c r="M16" s="56" t="n">
+        <v>287363128.490608</v>
+      </c>
+      <c r="N16" s="54" t="n"/>
+    </row>
+    <row r="17" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A17" s="62" t="inlineStr">
+        <is>
+          <t>Commercial margin%</t>
+        </is>
+      </c>
+      <c r="B17" s="63" t="n"/>
+      <c r="C17" s="63" t="n"/>
+      <c r="D17" s="63" t="n"/>
+      <c r="E17" s="63" t="n"/>
+      <c r="F17" s="63" t="n"/>
+      <c r="G17" s="63" t="n"/>
+      <c r="H17" s="63" t="n"/>
+      <c r="I17" s="63" t="n"/>
+      <c r="J17" s="63" t="n"/>
+      <c r="K17" s="63" t="n"/>
+      <c r="L17" s="63" t="n"/>
+      <c r="M17" s="63" t="n"/>
+      <c r="N17" s="54" t="n"/>
+    </row>
+    <row r="18" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A18" s="64" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
+      </c>
+      <c r="B18" s="56" t="n"/>
+      <c r="C18" s="56" t="n"/>
+      <c r="D18" s="56" t="n"/>
+      <c r="E18" s="56" t="n"/>
+      <c r="F18" s="56" t="n"/>
+      <c r="G18" s="56" t="n"/>
+      <c r="H18" s="56" t="n"/>
+      <c r="I18" s="56" t="n"/>
+      <c r="J18" s="56" t="n"/>
+      <c r="K18" s="56" t="n"/>
+      <c r="L18" s="56" t="n"/>
+      <c r="M18" s="56" t="n"/>
+      <c r="N18" s="54" t="n"/>
+    </row>
+    <row r="19" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A19" s="62" t="inlineStr">
+        <is>
+          <t>Losses%</t>
+        </is>
+      </c>
+      <c r="B19" s="63" t="n"/>
+      <c r="C19" s="63" t="n"/>
+      <c r="D19" s="63" t="n"/>
+      <c r="E19" s="63" t="n"/>
+      <c r="F19" s="63" t="n"/>
+      <c r="G19" s="63" t="n"/>
+      <c r="H19" s="63" t="n"/>
+      <c r="I19" s="63" t="n"/>
+      <c r="J19" s="63" t="n"/>
+      <c r="K19" s="63" t="n"/>
+      <c r="L19" s="63" t="n"/>
+      <c r="M19" s="63" t="n"/>
+      <c r="N19" s="54" t="n"/>
+    </row>
+    <row r="20" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A20" s="64" t="inlineStr">
+        <is>
+          <t>Logistics</t>
+        </is>
+      </c>
+      <c r="B20" s="56" t="n"/>
+      <c r="C20" s="56" t="n"/>
+      <c r="D20" s="56" t="n"/>
+      <c r="E20" s="56" t="n"/>
+      <c r="F20" s="56" t="n"/>
+      <c r="G20" s="56" t="n"/>
+      <c r="H20" s="56" t="n"/>
+      <c r="I20" s="56" t="n"/>
+      <c r="J20" s="56" t="n"/>
+      <c r="K20" s="56" t="n"/>
+      <c r="L20" s="56" t="n"/>
+      <c r="M20" s="56" t="n"/>
+      <c r="N20" s="54" t="n"/>
+    </row>
+    <row r="21" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A21" s="62" t="inlineStr">
+        <is>
+          <t>Logistics, %</t>
+        </is>
+      </c>
+      <c r="B21" s="63" t="n"/>
+      <c r="C21" s="63" t="n"/>
+      <c r="D21" s="63" t="n"/>
+      <c r="E21" s="63" t="n"/>
+      <c r="F21" s="63" t="n"/>
+      <c r="G21" s="63" t="n"/>
+      <c r="H21" s="63" t="n"/>
+      <c r="I21" s="63" t="n"/>
+      <c r="J21" s="63" t="n"/>
+      <c r="K21" s="63" t="n"/>
+      <c r="L21" s="63" t="n"/>
+      <c r="M21" s="63" t="n"/>
+      <c r="N21" s="54" t="n"/>
+    </row>
+    <row r="22" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A22" s="64" t="inlineStr">
+        <is>
+          <t>Stock provision</t>
+        </is>
+      </c>
+      <c r="B22" s="56" t="n"/>
+      <c r="C22" s="56" t="n"/>
+      <c r="D22" s="56" t="n"/>
+      <c r="E22" s="56" t="n"/>
+      <c r="F22" s="56" t="n"/>
+      <c r="G22" s="56" t="n"/>
+      <c r="H22" s="56" t="n"/>
+      <c r="I22" s="56" t="n"/>
+      <c r="J22" s="56" t="n"/>
+      <c r="K22" s="56" t="n"/>
+      <c r="L22" s="56" t="n"/>
+      <c r="M22" s="56" t="n"/>
+      <c r="N22" s="54" t="n"/>
+    </row>
+    <row r="23" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A23" s="62" t="inlineStr">
+        <is>
+          <t>Stock provision, %</t>
+        </is>
+      </c>
+      <c r="B23" s="63" t="n"/>
+      <c r="C23" s="63" t="n"/>
+      <c r="D23" s="63" t="n"/>
+      <c r="E23" s="63" t="n"/>
+      <c r="F23" s="63" t="n"/>
+      <c r="G23" s="63" t="n"/>
+      <c r="H23" s="63" t="n"/>
+      <c r="I23" s="63" t="n"/>
+      <c r="J23" s="63" t="n"/>
+      <c r="K23" s="63" t="n"/>
+      <c r="L23" s="63" t="n"/>
+      <c r="M23" s="63" t="n"/>
+      <c r="N23" s="54" t="n"/>
+    </row>
+    <row r="24" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A24" s="64" t="inlineStr">
+        <is>
+          <t>Packaging materials</t>
+        </is>
+      </c>
+      <c r="B24" s="56" t="n"/>
+      <c r="C24" s="56" t="n"/>
+      <c r="D24" s="56" t="n"/>
+      <c r="E24" s="56" t="n"/>
+      <c r="F24" s="56" t="n"/>
+      <c r="G24" s="56" t="n"/>
+      <c r="H24" s="56" t="n"/>
+      <c r="I24" s="56" t="n"/>
+      <c r="J24" s="56" t="n"/>
+      <c r="K24" s="56" t="n"/>
+      <c r="L24" s="56" t="n"/>
+      <c r="M24" s="56" t="n"/>
+      <c r="N24" s="54" t="n"/>
+    </row>
+    <row r="25" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A25" s="62" t="inlineStr">
+        <is>
+          <t>Packaging materials, %</t>
+        </is>
+      </c>
+      <c r="B25" s="63" t="n"/>
+      <c r="C25" s="63" t="n"/>
+      <c r="D25" s="63" t="n"/>
+      <c r="E25" s="63" t="n"/>
+      <c r="F25" s="63" t="n"/>
+      <c r="G25" s="63" t="n"/>
+      <c r="H25" s="63" t="n"/>
+      <c r="I25" s="63" t="n"/>
+      <c r="J25" s="63" t="n"/>
+      <c r="K25" s="63" t="n"/>
+      <c r="L25" s="63" t="n"/>
+      <c r="M25" s="63" t="n"/>
+      <c r="N25" s="54" t="n"/>
+    </row>
+    <row r="26" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A26" s="65" t="inlineStr">
+        <is>
+          <t>Gross margin</t>
+        </is>
+      </c>
+      <c r="B26" s="66" t="n">
+        <v>51397105.34437963</v>
+      </c>
+      <c r="C26" s="66" t="n">
+        <v>139325480.6976929</v>
+      </c>
+      <c r="D26" s="66" t="n">
+        <v>142508217.7192157</v>
+      </c>
+      <c r="E26" s="66" t="n">
+        <v>74530640.26743269</v>
+      </c>
+      <c r="F26" s="66" t="n">
+        <v>290925019.5202637</v>
+      </c>
+      <c r="G26" s="66" t="n">
+        <v>342575263.6328037</v>
+      </c>
+      <c r="H26" s="66" t="n">
+        <v>143329946.9682095</v>
+      </c>
+      <c r="I26" s="66" t="n">
+        <v>177328700.0704224</v>
+      </c>
+      <c r="J26" s="66" t="n">
+        <v>335398417.4200364</v>
+      </c>
+      <c r="K26" s="66" t="n">
+        <v>87471840.42115504</v>
+      </c>
+      <c r="L26" s="66" t="n">
+        <v>211633363.2039606</v>
+      </c>
+      <c r="M26" s="66" t="n">
+        <v>287363128.490608</v>
+      </c>
+      <c r="N26" s="54" t="n"/>
+    </row>
+    <row r="27" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A27" s="67" t="inlineStr">
+        <is>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="B27" s="68" t="n"/>
+      <c r="C27" s="68" t="n"/>
+      <c r="D27" s="68" t="n"/>
+      <c r="E27" s="68" t="n"/>
+      <c r="F27" s="68" t="n"/>
+      <c r="G27" s="68" t="n"/>
+      <c r="H27" s="68" t="n"/>
+      <c r="I27" s="68" t="n"/>
+      <c r="J27" s="68" t="n"/>
+      <c r="K27" s="68" t="n"/>
+      <c r="L27" s="68" t="n"/>
+      <c r="M27" s="68" t="n"/>
+      <c r="N27" s="54" t="n"/>
+    </row>
+    <row r="28" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A28" s="64" t="inlineStr">
+        <is>
+          <t>Total other revenue</t>
+        </is>
+      </c>
+      <c r="B28" s="56" t="n"/>
+      <c r="C28" s="56" t="n"/>
+      <c r="D28" s="56" t="n"/>
+      <c r="E28" s="56" t="n"/>
+      <c r="F28" s="56" t="n"/>
+      <c r="G28" s="56" t="n"/>
+      <c r="H28" s="56" t="n"/>
+      <c r="I28" s="56" t="n"/>
+      <c r="J28" s="56" t="n"/>
+      <c r="K28" s="56" t="n"/>
+      <c r="L28" s="56" t="n"/>
+      <c r="M28" s="56" t="n"/>
+      <c r="N28" s="54" t="n"/>
+    </row>
+    <row r="29" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A29" s="62" t="inlineStr">
+        <is>
+          <t>Total other revenue %</t>
+        </is>
+      </c>
+      <c r="B29" s="63" t="n"/>
+      <c r="C29" s="63" t="n"/>
+      <c r="D29" s="63" t="n"/>
+      <c r="E29" s="63" t="n"/>
+      <c r="F29" s="63" t="n"/>
+      <c r="G29" s="63" t="n"/>
+      <c r="H29" s="63" t="n"/>
+      <c r="I29" s="63" t="n"/>
+      <c r="J29" s="63" t="n"/>
+      <c r="K29" s="63" t="n"/>
+      <c r="L29" s="63" t="n"/>
+      <c r="M29" s="63" t="n"/>
+      <c r="N29" s="54" t="n"/>
+    </row>
+    <row r="30" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A30" s="69" t="inlineStr">
+        <is>
+          <t>Total OPEX</t>
+        </is>
+      </c>
+      <c r="B30" s="70" t="n">
+        <v>-96813784.15000001</v>
+      </c>
+      <c r="C30" s="70" t="n">
+        <v>-97507146.21000001</v>
+      </c>
+      <c r="D30" s="70" t="n">
+        <v>-96245068.84020025</v>
+      </c>
+      <c r="E30" s="70" t="n">
+        <v>-106548011.4808188</v>
+      </c>
+      <c r="F30" s="70" t="n">
+        <v>-122810011.2396875</v>
+      </c>
+      <c r="G30" s="70" t="n">
+        <v>-148674397.1935303</v>
+      </c>
+      <c r="H30" s="70" t="n">
+        <v>-106802888.06466</v>
+      </c>
+      <c r="I30" s="70" t="n">
+        <v>-128491903.638262</v>
+      </c>
+      <c r="J30" s="70" t="n">
+        <v>24999360.40751434</v>
+      </c>
+      <c r="K30" s="70" t="n">
+        <v>-126571937.7488332</v>
+      </c>
+      <c r="L30" s="70" t="n">
+        <v>-129770864.6887665</v>
+      </c>
+      <c r="M30" s="70" t="n">
+        <v>-129977288.999939</v>
+      </c>
+      <c r="N30" s="54" t="n"/>
+    </row>
+    <row r="31" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A31" s="71" t="inlineStr">
+        <is>
+          <t>Total OPEX %</t>
+        </is>
+      </c>
+      <c r="B31" s="72" t="n"/>
+      <c r="C31" s="72" t="n"/>
+      <c r="D31" s="72" t="n"/>
+      <c r="E31" s="72" t="n"/>
+      <c r="F31" s="72" t="n"/>
+      <c r="G31" s="72" t="n"/>
+      <c r="H31" s="72" t="n"/>
+      <c r="I31" s="72" t="n"/>
+      <c r="J31" s="72" t="n"/>
+      <c r="K31" s="72" t="n"/>
+      <c r="L31" s="72" t="n"/>
+      <c r="M31" s="72" t="n"/>
+      <c r="N31" s="54" t="n"/>
+    </row>
+    <row r="32" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A32" s="64" t="inlineStr">
+        <is>
+          <t>PEX</t>
+        </is>
+      </c>
+      <c r="B32" s="56" t="n">
+        <v>-95938090.5</v>
+      </c>
+      <c r="C32" s="56" t="n">
+        <v>-95034802.90000001</v>
+      </c>
+      <c r="D32" s="56" t="n">
+        <v>-96333821.15020025</v>
+      </c>
+      <c r="E32" s="56" t="n">
+        <v>-103523767.9508188</v>
+      </c>
+      <c r="F32" s="56" t="n">
+        <v>-113707319.5496875</v>
+      </c>
+      <c r="G32" s="56" t="n">
+        <v>-122657190.2135303</v>
+      </c>
+      <c r="H32" s="56" t="n">
+        <v>-99072375.46466005</v>
+      </c>
+      <c r="I32" s="56" t="n">
+        <v>-114474730.038262</v>
+      </c>
+      <c r="J32" s="56" t="n">
+        <v>44410155.00751434</v>
+      </c>
+      <c r="K32" s="56" t="n">
+        <v>-115782938.2760877</v>
+      </c>
+      <c r="L32" s="56" t="n">
+        <v>-115653214.4132013</v>
+      </c>
+      <c r="M32" s="56" t="n">
+        <v>-115475622.9761398</v>
+      </c>
+      <c r="N32" s="54" t="n"/>
+    </row>
+    <row r="33" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A33" s="62" t="inlineStr">
+        <is>
+          <t>PEX%</t>
+        </is>
+      </c>
+      <c r="B33" s="73" t="n"/>
+      <c r="C33" s="73" t="n"/>
+      <c r="D33" s="73" t="n"/>
+      <c r="E33" s="73" t="n"/>
+      <c r="F33" s="73" t="n"/>
+      <c r="G33" s="73" t="n"/>
+      <c r="H33" s="73" t="n"/>
+      <c r="I33" s="73" t="n"/>
+      <c r="J33" s="73" t="n"/>
+      <c r="K33" s="73" t="n"/>
+      <c r="L33" s="73" t="n"/>
+      <c r="M33" s="73" t="n"/>
+      <c r="N33" s="54" t="n"/>
+    </row>
+    <row r="34" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A34" s="62" t="inlineStr">
+        <is>
+          <t>PEX retail</t>
+        </is>
+      </c>
+      <c r="B34" s="74" t="n"/>
+      <c r="C34" s="74" t="n"/>
+      <c r="D34" s="74" t="n"/>
+      <c r="E34" s="74" t="n"/>
+      <c r="F34" s="74" t="n"/>
+      <c r="G34" s="74" t="n"/>
+      <c r="H34" s="74" t="n"/>
+      <c r="I34" s="74" t="n"/>
+      <c r="J34" s="74" t="n"/>
+      <c r="K34" s="74" t="n"/>
+      <c r="L34" s="74" t="n"/>
+      <c r="M34" s="74" t="n"/>
+      <c r="N34" s="54" t="n"/>
+    </row>
+    <row r="35" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A35" s="62" t="inlineStr">
+        <is>
+          <t>PEX admin</t>
+        </is>
+      </c>
+      <c r="B35" s="56" t="n">
+        <v>-92886360.5</v>
+      </c>
+      <c r="C35" s="56" t="n">
+        <v>-94592513.90000001</v>
+      </c>
+      <c r="D35" s="56" t="n">
+        <v>-95109178.44724879</v>
+      </c>
+      <c r="E35" s="56" t="n">
+        <v>-101882236.5107256</v>
+      </c>
+      <c r="F35" s="56" t="n">
+        <v>-112467620.9260646</v>
+      </c>
+      <c r="G35" s="56" t="n">
+        <v>-106240266.7461649</v>
+      </c>
+      <c r="H35" s="56" t="n">
+        <v>-101336835.3946933</v>
+      </c>
+      <c r="I35" s="56" t="n">
+        <v>-111304741.7725611</v>
+      </c>
+      <c r="J35" s="56" t="n">
+        <v>44821201.26104592</v>
+      </c>
+      <c r="K35" s="56" t="n">
+        <v>-111510282.7511398</v>
+      </c>
+      <c r="L35" s="56" t="n">
+        <v>-111510282.7511398</v>
+      </c>
+      <c r="M35" s="56" t="n">
+        <v>-111510282.7511398</v>
+      </c>
+      <c r="N35" s="54" t="n"/>
+    </row>
+    <row r="36" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A36" s="62" t="inlineStr">
+        <is>
+          <t>PEX other</t>
+        </is>
+      </c>
+      <c r="B36" s="61" t="n">
+        <v>-3051730</v>
+      </c>
+      <c r="C36" s="61" t="n">
+        <v>-442289</v>
+      </c>
+      <c r="D36" s="61" t="n">
+        <v>-1224642.702951454</v>
+      </c>
+      <c r="E36" s="61" t="n">
+        <v>-1641531.440093187</v>
+      </c>
+      <c r="F36" s="61" t="n">
+        <v>-1239698.623622975</v>
+      </c>
+      <c r="G36" s="61" t="n">
+        <v>-16416923.46736547</v>
+      </c>
+      <c r="H36" s="61" t="n">
+        <v>2264459.930033199</v>
+      </c>
+      <c r="I36" s="61" t="n">
+        <v>-3169988.265700941</v>
+      </c>
+      <c r="J36" s="61" t="n">
+        <v>-411046.2535315827</v>
+      </c>
+      <c r="K36" s="61" t="n">
+        <v>-4272655.524947914</v>
+      </c>
+      <c r="L36" s="61" t="n">
+        <v>-4142931.662061526</v>
+      </c>
+      <c r="M36" s="61" t="n">
+        <v>-3965340.224999997</v>
+      </c>
+      <c r="N36" s="54" t="n"/>
+    </row>
+    <row r="37" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A37" s="64" t="inlineStr">
+        <is>
+          <t>NON PEX</t>
+        </is>
+      </c>
+      <c r="B37" s="75" t="n">
+        <v>-875693.65</v>
+      </c>
+      <c r="C37" s="75" t="n">
+        <v>-2472343.31</v>
+      </c>
+      <c r="D37" s="75" t="n">
+        <v>88752.30999999994</v>
+      </c>
+      <c r="E37" s="75" t="n">
+        <v>-3024243.53</v>
+      </c>
+      <c r="F37" s="75" t="n">
+        <v>-9102691.690000001</v>
+      </c>
+      <c r="G37" s="75" t="n">
+        <v>-26017206.98</v>
+      </c>
+      <c r="H37" s="75" t="n">
+        <v>-7730512.6</v>
+      </c>
+      <c r="I37" s="75" t="n">
+        <v>-14017173.6</v>
+      </c>
+      <c r="J37" s="75" t="n">
+        <v>-19410794.6</v>
+      </c>
+      <c r="K37" s="75" t="n">
+        <v>-10788999.47274554</v>
+      </c>
+      <c r="L37" s="75" t="n">
+        <v>-14117650.27556517</v>
+      </c>
+      <c r="M37" s="75" t="n">
+        <v>-14501666.02379919</v>
+      </c>
+      <c r="N37" s="54" t="n"/>
+    </row>
+    <row r="38" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A38" s="76" t="inlineStr">
+        <is>
+          <t>NON PEX%</t>
+        </is>
+      </c>
+      <c r="B38" s="73" t="n"/>
+      <c r="C38" s="73" t="n"/>
+      <c r="D38" s="73" t="n"/>
+      <c r="E38" s="73" t="n"/>
+      <c r="F38" s="73" t="n"/>
+      <c r="G38" s="73" t="n"/>
+      <c r="H38" s="73" t="n"/>
+      <c r="I38" s="73" t="n"/>
+      <c r="J38" s="73" t="n"/>
+      <c r="K38" s="73" t="n"/>
+      <c r="L38" s="73" t="n"/>
+      <c r="M38" s="73" t="n"/>
+      <c r="N38" s="54" t="n"/>
+    </row>
+    <row r="39" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A39" s="64" t="inlineStr">
+        <is>
+          <t>Picking and Delivery</t>
+        </is>
+      </c>
+      <c r="B39" s="58" t="n"/>
+      <c r="C39" s="58" t="n"/>
+      <c r="D39" s="58" t="n"/>
+      <c r="E39" s="58" t="n"/>
+      <c r="F39" s="58" t="n"/>
+      <c r="G39" s="58" t="n"/>
+      <c r="H39" s="58" t="n"/>
+      <c r="I39" s="58" t="n"/>
+      <c r="J39" s="58" t="n"/>
+      <c r="K39" s="58" t="n"/>
+      <c r="L39" s="58" t="n"/>
+      <c r="M39" s="58" t="n"/>
+      <c r="N39" s="54" t="n"/>
+    </row>
+    <row r="40" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A40" s="62" t="inlineStr">
+        <is>
+          <t>Picking and Delivery, %</t>
+        </is>
+      </c>
+      <c r="B40" s="63" t="n"/>
+      <c r="C40" s="63" t="n"/>
+      <c r="D40" s="63" t="n"/>
+      <c r="E40" s="63" t="n"/>
+      <c r="F40" s="63" t="n"/>
+      <c r="G40" s="63" t="n"/>
+      <c r="H40" s="63" t="n"/>
+      <c r="I40" s="63" t="n"/>
+      <c r="J40" s="63" t="n"/>
+      <c r="K40" s="63" t="n"/>
+      <c r="L40" s="63" t="n"/>
+      <c r="M40" s="63" t="n"/>
+      <c r="N40" s="54" t="n"/>
+    </row>
+    <row r="41" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A41" s="64" t="inlineStr">
+        <is>
+          <t>Utilities costs</t>
+        </is>
+      </c>
+      <c r="B41" s="56" t="n"/>
+      <c r="C41" s="56" t="n"/>
+      <c r="D41" s="56" t="n"/>
+      <c r="E41" s="56" t="n"/>
+      <c r="F41" s="56" t="n"/>
+      <c r="G41" s="56" t="n"/>
+      <c r="H41" s="56" t="n"/>
+      <c r="I41" s="56" t="n"/>
+      <c r="J41" s="56" t="n"/>
+      <c r="K41" s="56" t="n"/>
+      <c r="L41" s="56" t="n"/>
+      <c r="M41" s="56" t="n"/>
+      <c r="N41" s="54" t="n"/>
+    </row>
+    <row r="42" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A42" s="62" t="inlineStr">
+        <is>
+          <t>Utilities costs, %</t>
+        </is>
+      </c>
+      <c r="B42" s="73" t="n"/>
+      <c r="C42" s="73" t="n"/>
+      <c r="D42" s="73" t="n"/>
+      <c r="E42" s="73" t="n"/>
+      <c r="F42" s="73" t="n"/>
+      <c r="G42" s="73" t="n"/>
+      <c r="H42" s="73" t="n"/>
+      <c r="I42" s="73" t="n"/>
+      <c r="J42" s="73" t="n"/>
+      <c r="K42" s="73" t="n"/>
+      <c r="L42" s="73" t="n"/>
+      <c r="M42" s="73" t="n"/>
+      <c r="N42" s="54" t="n"/>
+    </row>
+    <row r="43" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A43" s="64" t="inlineStr">
+        <is>
+          <t>Repair and maintenance</t>
+        </is>
+      </c>
+      <c r="B43" s="58" t="n"/>
+      <c r="C43" s="58" t="n"/>
+      <c r="D43" s="58" t="n"/>
+      <c r="E43" s="58" t="n"/>
+      <c r="F43" s="58" t="n"/>
+      <c r="G43" s="58" t="n"/>
+      <c r="H43" s="58" t="n"/>
+      <c r="I43" s="58" t="n"/>
+      <c r="J43" s="58" t="n"/>
+      <c r="K43" s="58" t="n"/>
+      <c r="L43" s="58" t="n"/>
+      <c r="M43" s="58" t="n"/>
+      <c r="N43" s="54" t="n"/>
+    </row>
+    <row r="44" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A44" s="62" t="inlineStr">
+        <is>
+          <t>Repair and maintenance, %</t>
+        </is>
+      </c>
+      <c r="B44" s="73" t="n"/>
+      <c r="C44" s="73" t="n"/>
+      <c r="D44" s="73" t="n"/>
+      <c r="E44" s="73" t="n"/>
+      <c r="F44" s="73" t="n"/>
+      <c r="G44" s="73" t="n"/>
+      <c r="H44" s="73" t="n"/>
+      <c r="I44" s="73" t="n"/>
+      <c r="J44" s="73" t="n"/>
+      <c r="K44" s="73" t="n"/>
+      <c r="L44" s="73" t="n"/>
+      <c r="M44" s="73" t="n"/>
+      <c r="N44" s="54" t="n"/>
+    </row>
+    <row r="45" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A45" s="64" t="inlineStr">
+        <is>
+          <t>Packaging and materials</t>
+        </is>
+      </c>
+      <c r="B45" s="58" t="n"/>
+      <c r="C45" s="58" t="n"/>
+      <c r="D45" s="58" t="n"/>
+      <c r="E45" s="58" t="n"/>
+      <c r="F45" s="58" t="n"/>
+      <c r="G45" s="58" t="n"/>
+      <c r="H45" s="58" t="n"/>
+      <c r="I45" s="58" t="n"/>
+      <c r="J45" s="58" t="n"/>
+      <c r="K45" s="58" t="n"/>
+      <c r="L45" s="58" t="n"/>
+      <c r="M45" s="58" t="n"/>
+      <c r="N45" s="54" t="n"/>
+    </row>
+    <row r="46" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A46" s="62" t="inlineStr">
+        <is>
+          <t>Packaging and materials, %</t>
+        </is>
+      </c>
+      <c r="B46" s="73" t="n"/>
+      <c r="C46" s="73" t="n"/>
+      <c r="D46" s="73" t="n"/>
+      <c r="E46" s="73" t="n"/>
+      <c r="F46" s="73" t="n"/>
+      <c r="G46" s="73" t="n"/>
+      <c r="H46" s="73" t="n"/>
+      <c r="I46" s="73" t="n"/>
+      <c r="J46" s="73" t="n"/>
+      <c r="K46" s="73" t="n"/>
+      <c r="L46" s="73" t="n"/>
+      <c r="M46" s="73" t="n"/>
+      <c r="N46" s="54" t="n"/>
+    </row>
+    <row r="47" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A47" s="64" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+      <c r="B47" s="56" t="n"/>
+      <c r="C47" s="56" t="n"/>
+      <c r="D47" s="56" t="n"/>
+      <c r="E47" s="56" t="n"/>
+      <c r="F47" s="56" t="n"/>
+      <c r="G47" s="56" t="n"/>
+      <c r="H47" s="56" t="n"/>
+      <c r="I47" s="56" t="n"/>
+      <c r="J47" s="56" t="n"/>
+      <c r="K47" s="56" t="n"/>
+      <c r="L47" s="56" t="n"/>
+      <c r="M47" s="56" t="n"/>
+      <c r="N47" s="54" t="n"/>
+    </row>
+    <row r="48" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A48" s="62" t="inlineStr">
+        <is>
+          <t>Security, %</t>
+        </is>
+      </c>
+      <c r="B48" s="73" t="n"/>
+      <c r="C48" s="73" t="n"/>
+      <c r="D48" s="73" t="n"/>
+      <c r="E48" s="73" t="n"/>
+      <c r="F48" s="73" t="n"/>
+      <c r="G48" s="73" t="n"/>
+      <c r="H48" s="73" t="n"/>
+      <c r="I48" s="73" t="n"/>
+      <c r="J48" s="73" t="n"/>
+      <c r="K48" s="73" t="n"/>
+      <c r="L48" s="73" t="n"/>
+      <c r="M48" s="73" t="n"/>
+      <c r="N48" s="54" t="n"/>
+    </row>
+    <row r="49" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A49" s="77" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B49" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="56" t="n">
+        <v>-983250</v>
+      </c>
+      <c r="F49" s="56" t="n">
+        <v>-6535146.83</v>
+      </c>
+      <c r="G49" s="56" t="n">
+        <v>-11434752.42</v>
+      </c>
+      <c r="H49" s="56" t="n">
+        <v>-2230389.29</v>
+      </c>
+      <c r="I49" s="56" t="n">
+        <v>-6713829.45</v>
+      </c>
+      <c r="J49" s="56" t="n">
+        <v>-6400104.62</v>
+      </c>
+      <c r="K49" s="56" t="n">
+        <v>-4418658.333333334</v>
+      </c>
+      <c r="L49" s="56" t="n">
+        <v>-7118658.333333334</v>
+      </c>
+      <c r="M49" s="56" t="n">
+        <v>-5918658.333333334</v>
+      </c>
+      <c r="N49" s="54" t="n"/>
+    </row>
+    <row r="50" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A50" s="57" t="inlineStr">
+        <is>
+          <t>Own Marketing</t>
+        </is>
+      </c>
+      <c r="B50" s="78" t="n"/>
+      <c r="C50" s="78" t="n"/>
+      <c r="D50" s="78" t="n"/>
+      <c r="E50" s="78" t="n"/>
+      <c r="F50" s="78" t="n"/>
+      <c r="G50" s="78" t="n"/>
+      <c r="H50" s="78" t="n"/>
+      <c r="I50" s="78" t="n"/>
+      <c r="J50" s="78" t="n"/>
+      <c r="K50" s="78" t="n"/>
+      <c r="L50" s="78" t="n"/>
+      <c r="M50" s="78" t="n"/>
+      <c r="N50" s="54" t="n"/>
+    </row>
+    <row r="51" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A51" s="57" t="inlineStr">
+        <is>
+          <t>Partners' Marketing</t>
+        </is>
+      </c>
+      <c r="B51" s="74" t="n"/>
+      <c r="C51" s="74" t="n"/>
+      <c r="D51" s="74" t="n"/>
+      <c r="E51" s="74" t="n"/>
+      <c r="F51" s="74" t="n"/>
+      <c r="G51" s="74" t="n"/>
+      <c r="H51" s="74" t="n"/>
+      <c r="I51" s="74" t="n"/>
+      <c r="J51" s="74" t="n"/>
+      <c r="K51" s="74" t="n"/>
+      <c r="L51" s="74" t="n"/>
+      <c r="M51" s="74" t="n"/>
+      <c r="N51" s="54" t="n"/>
+    </row>
+    <row r="52" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A52" s="79" t="inlineStr">
+        <is>
+          <t>Marketing, %</t>
+        </is>
+      </c>
+      <c r="B52" s="73" t="n"/>
+      <c r="C52" s="73" t="n"/>
+      <c r="D52" s="73" t="n"/>
+      <c r="E52" s="73" t="n"/>
+      <c r="F52" s="73" t="n"/>
+      <c r="G52" s="73" t="n"/>
+      <c r="H52" s="73" t="n"/>
+      <c r="I52" s="73" t="n"/>
+      <c r="J52" s="73" t="n"/>
+      <c r="K52" s="73" t="n"/>
+      <c r="L52" s="73" t="n"/>
+      <c r="M52" s="73" t="n"/>
+      <c r="N52" s="54" t="n"/>
+    </row>
+    <row r="53" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A53" s="77" t="inlineStr">
+        <is>
+          <t>Consulting and insurance</t>
+        </is>
+      </c>
+      <c r="B53" s="58" t="n">
+        <v>-155854</v>
+      </c>
+      <c r="C53" s="58" t="n">
+        <v>-1633817</v>
+      </c>
+      <c r="D53" s="58" t="n">
+        <v>772474.76</v>
+      </c>
+      <c r="E53" s="58" t="n">
+        <v>-1371206.32</v>
+      </c>
+      <c r="F53" s="58" t="n">
+        <v>-2464153.540000001</v>
+      </c>
+      <c r="G53" s="58" t="n">
+        <v>-2164074.739999998</v>
+      </c>
+      <c r="H53" s="58" t="n">
+        <v>-940167.4499999998</v>
+      </c>
+      <c r="I53" s="58" t="n">
+        <v>-964293.23</v>
+      </c>
+      <c r="J53" s="58" t="n">
+        <v>-3887514.700000001</v>
+      </c>
+      <c r="K53" s="58" t="n">
+        <v>-1283507.24</v>
+      </c>
+      <c r="L53" s="58" t="n">
+        <v>-1283507.24</v>
+      </c>
+      <c r="M53" s="58" t="n">
+        <v>-1283507.24</v>
+      </c>
+      <c r="N53" s="54" t="n"/>
+    </row>
+    <row r="54" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A54" s="79" t="inlineStr">
+        <is>
+          <t>Consulting and insurance, %</t>
+        </is>
+      </c>
+      <c r="B54" s="73" t="n"/>
+      <c r="C54" s="73" t="n"/>
+      <c r="D54" s="73" t="n"/>
+      <c r="E54" s="73" t="n"/>
+      <c r="F54" s="73" t="n"/>
+      <c r="G54" s="73" t="n"/>
+      <c r="H54" s="73" t="n"/>
+      <c r="I54" s="73" t="n"/>
+      <c r="J54" s="73" t="n"/>
+      <c r="K54" s="73" t="n"/>
+      <c r="L54" s="73" t="n"/>
+      <c r="M54" s="73" t="n"/>
+      <c r="N54" s="54" t="n"/>
+    </row>
+    <row r="55" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A55" s="64" t="inlineStr">
+        <is>
+          <t>Other OPEX</t>
+        </is>
+      </c>
+      <c r="B55" s="56" t="n">
+        <v>-719839.65</v>
+      </c>
+      <c r="C55" s="56" t="n">
+        <v>-838526.3100000001</v>
+      </c>
+      <c r="D55" s="56" t="n">
+        <v>-683722.4500000001</v>
+      </c>
+      <c r="E55" s="56" t="n">
+        <v>-669787.2100000001</v>
+      </c>
+      <c r="F55" s="56" t="n">
+        <v>-103391.3200000003</v>
+      </c>
+      <c r="G55" s="56" t="n">
+        <v>-12418379.82</v>
+      </c>
+      <c r="H55" s="56" t="n">
+        <v>-4559955.859999999</v>
+      </c>
+      <c r="I55" s="56" t="n">
+        <v>-6339050.920000001</v>
+      </c>
+      <c r="J55" s="56" t="n">
+        <v>-9123175.279999999</v>
+      </c>
+      <c r="K55" s="56" t="n">
+        <v>-5086833.899412203</v>
+      </c>
+      <c r="L55" s="56" t="n">
+        <v>-5715484.70223184</v>
+      </c>
+      <c r="M55" s="56" t="n">
+        <v>-7299500.450465856</v>
+      </c>
+      <c r="N55" s="54" t="n"/>
+    </row>
+    <row r="56" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A56" s="76" t="inlineStr">
+        <is>
+          <t>Other OPEX, %</t>
+        </is>
+      </c>
+      <c r="B56" s="80" t="n"/>
+      <c r="C56" s="80" t="n"/>
+      <c r="D56" s="80" t="n"/>
+      <c r="E56" s="80" t="n"/>
+      <c r="F56" s="80" t="n"/>
+      <c r="G56" s="80" t="n"/>
+      <c r="H56" s="80" t="n"/>
+      <c r="I56" s="80" t="n"/>
+      <c r="J56" s="80" t="n"/>
+      <c r="K56" s="80" t="n"/>
+      <c r="L56" s="80" t="n"/>
+      <c r="M56" s="80" t="n"/>
+      <c r="N56" s="54" t="n"/>
+    </row>
+    <row r="57" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A57" s="64" t="inlineStr">
+        <is>
+          <t>Rent</t>
+        </is>
+      </c>
+      <c r="B57" s="56" t="n"/>
+      <c r="C57" s="56" t="n"/>
+      <c r="D57" s="56" t="n"/>
+      <c r="E57" s="56" t="n"/>
+      <c r="F57" s="56" t="n"/>
+      <c r="G57" s="56" t="n"/>
+      <c r="H57" s="56" t="n"/>
+      <c r="I57" s="56" t="n"/>
+      <c r="J57" s="56" t="n"/>
+      <c r="K57" s="56" t="n"/>
+      <c r="L57" s="56" t="n"/>
+      <c r="M57" s="56" t="n"/>
+      <c r="N57" s="54" t="n"/>
+    </row>
+    <row r="58" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A58" s="62" t="inlineStr">
+        <is>
+          <t>Rent %</t>
+        </is>
+      </c>
+      <c r="B58" s="73" t="n"/>
+      <c r="C58" s="73" t="n"/>
+      <c r="D58" s="73" t="n"/>
+      <c r="E58" s="73" t="n"/>
+      <c r="F58" s="73" t="n"/>
+      <c r="G58" s="73" t="n"/>
+      <c r="H58" s="73" t="n"/>
+      <c r="I58" s="73" t="n"/>
+      <c r="J58" s="73" t="n"/>
+      <c r="K58" s="73" t="n"/>
+      <c r="L58" s="73" t="n"/>
+      <c r="M58" s="73" t="n"/>
+      <c r="N58" s="54" t="n"/>
+    </row>
+    <row r="59" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A59" s="81" t="inlineStr">
+        <is>
+          <t>LTI</t>
+        </is>
+      </c>
+      <c r="B59" s="82" t="n"/>
+      <c r="C59" s="82" t="n"/>
+      <c r="D59" s="82" t="n"/>
+      <c r="E59" s="82" t="n"/>
+      <c r="F59" s="82" t="n"/>
+      <c r="G59" s="82" t="n"/>
+      <c r="H59" s="82" t="n"/>
+      <c r="I59" s="82" t="n"/>
+      <c r="J59" s="82" t="n"/>
+      <c r="K59" s="82" t="n"/>
+      <c r="L59" s="82" t="n"/>
+      <c r="M59" s="82" t="n"/>
+      <c r="N59" s="54" t="n"/>
+    </row>
+    <row r="60" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A60" s="65" t="inlineStr">
+        <is>
+          <t xml:space="preserve">EBITDA </t>
+        </is>
+      </c>
+      <c r="B60" s="66" t="n">
+        <v>-45416678.80562037</v>
+      </c>
+      <c r="C60" s="66" t="n">
+        <v>41818334.48769289</v>
+      </c>
+      <c r="D60" s="66" t="n">
+        <v>46263148.87901545</v>
+      </c>
+      <c r="E60" s="66" t="n">
+        <v>-32017371.21338612</v>
+      </c>
+      <c r="F60" s="66" t="n">
+        <v>168115008.2805762</v>
+      </c>
+      <c r="G60" s="66" t="n">
+        <v>193900866.4392734</v>
+      </c>
+      <c r="H60" s="66" t="n">
+        <v>36527058.90354946</v>
+      </c>
+      <c r="I60" s="66" t="n">
+        <v>48836796.43216041</v>
+      </c>
+      <c r="J60" s="66" t="n">
+        <v>360397777.8275507</v>
+      </c>
+      <c r="K60" s="66" t="n">
+        <v>-39100097.3276782</v>
+      </c>
+      <c r="L60" s="66" t="n">
+        <v>81862498.51519412</v>
+      </c>
+      <c r="M60" s="66" t="n">
+        <v>157385839.490669</v>
+      </c>
+      <c r="N60" s="54" t="n"/>
+    </row>
+    <row r="61" hidden="1" ht="15" customFormat="1" customHeight="1" s="51">
+      <c r="A61" s="83" t="inlineStr">
+        <is>
+          <t>EBITDA, %</t>
+        </is>
+      </c>
+      <c r="B61" s="84" t="n"/>
+      <c r="C61" s="84" t="n"/>
+      <c r="D61" s="84" t="n"/>
+      <c r="E61" s="84" t="n"/>
+      <c r="F61" s="84" t="n"/>
+      <c r="G61" s="84" t="n"/>
+      <c r="H61" s="84" t="n"/>
+      <c r="I61" s="84" t="n"/>
+      <c r="J61" s="84" t="n"/>
+      <c r="K61" s="84" t="n"/>
+      <c r="L61" s="84" t="n"/>
+      <c r="M61" s="84" t="n"/>
+      <c r="N61" s="54" t="n"/>
+    </row>
+    <row r="63" ht="15" customHeight="1" s="48">
+      <c r="B63" s="85" t="n"/>
+      <c r="C63" s="85" t="n"/>
+      <c r="D63" s="85" t="n"/>
+      <c r="E63" s="85" t="n"/>
+      <c r="F63" s="85" t="n"/>
+      <c r="G63" s="85" t="n"/>
+      <c r="H63" s="85" t="n"/>
+      <c r="I63" s="85" t="n"/>
+      <c r="J63" s="85" t="n"/>
+      <c r="K63" s="85" t="n"/>
+      <c r="L63" s="85" t="n"/>
+      <c r="M63" s="85" t="n"/>
+    </row>
+    <row r="64" ht="15" customHeight="1" s="48">
+      <c r="B64" s="86" t="n"/>
+      <c r="C64" s="86" t="n"/>
+      <c r="D64" s="86" t="n"/>
+      <c r="E64" s="86" t="n"/>
+      <c r="F64" s="86" t="n"/>
+      <c r="G64" s="86" t="n"/>
+      <c r="H64" s="86" t="n"/>
+      <c r="I64" s="86" t="n"/>
+      <c r="J64" s="86" t="n"/>
+      <c r="K64" s="86" t="n"/>
+      <c r="L64" s="86" t="n"/>
+      <c r="M64" s="86" t="n"/>
+    </row>
+  </sheetData>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="58" customWidth="1" style="48" min="1" max="1"/>
+    <col width="11" customWidth="1" style="48" min="2" max="2"/>
+    <col width="11" customWidth="1" style="48" min="3" max="3"/>
+    <col width="11" customWidth="1" style="48" min="4" max="4"/>
+    <col width="11" customWidth="1" style="48" min="5" max="5"/>
+    <col width="11" customWidth="1" style="48" min="6" max="6"/>
+    <col width="11" customWidth="1" style="48" min="7" max="7"/>
+    <col width="11" customWidth="1" style="48" min="8" max="8"/>
+    <col width="11" customWidth="1" style="48" min="9" max="9"/>
+    <col width="11" customWidth="1" style="48" min="10" max="10"/>
+    <col width="11" customWidth="1" style="48" min="11" max="11"/>
+    <col width="11" customWidth="1" style="48" min="12" max="12"/>
+    <col width="11" customWidth="1" style="48" min="13" max="13"/>
+    <col width="11" customWidth="1" style="48" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="87" t="inlineStr">
+        <is>
+          <t>Свод 2026 в новой логике, млн руб. База: выгрузка «Adtech_прогноз 9+3 для конс» от 14.10 (факт янв–сен, прогноз окт–дек)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="46" t="inlineStr">
+        <is>
+          <t>Новая логика: закупка трафика (расходы на маркетинг в сети интернет) перенесена из Marketing в Commercial margin. Commercial margin = инкремент выручки без E-comm за вычетом всех расходов, привязанных к выручке: вознаграждения РА и блогерам (как и раньше) и закупка трафика. EBITDA не меняется.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="88" t="inlineStr">
+        <is>
+          <t>Статья</t>
+        </is>
+      </c>
+      <c r="B4" s="88" t="inlineStr">
+        <is>
+          <t>jan'26</t>
+        </is>
+      </c>
+      <c r="C4" s="88" t="inlineStr">
+        <is>
+          <t>feb'26</t>
+        </is>
+      </c>
+      <c r="D4" s="88" t="inlineStr">
+        <is>
+          <t>mar'26</t>
+        </is>
+      </c>
+      <c r="E4" s="88" t="inlineStr">
+        <is>
+          <t>apr'26</t>
+        </is>
+      </c>
+      <c r="F4" s="88" t="inlineStr">
+        <is>
+          <t>may'26</t>
+        </is>
+      </c>
+      <c r="G4" s="88" t="inlineStr">
+        <is>
+          <t>jun'26</t>
+        </is>
+      </c>
+      <c r="H4" s="88" t="inlineStr">
+        <is>
+          <t>jul'26</t>
+        </is>
+      </c>
+      <c r="I4" s="88" t="inlineStr">
+        <is>
+          <t>aug'26</t>
+        </is>
+      </c>
+      <c r="J4" s="88" t="inlineStr">
+        <is>
+          <t>sep'26</t>
+        </is>
+      </c>
+      <c r="K4" s="88" t="inlineStr">
+        <is>
+          <t>oct'26</t>
+        </is>
+      </c>
+      <c r="L4" s="88" t="inlineStr">
+        <is>
+          <t>nov'26</t>
+        </is>
+      </c>
+      <c r="M4" s="88" t="inlineStr">
+        <is>
+          <t>dec'26</t>
+        </is>
+      </c>
+      <c r="N4" s="88" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="87" t="inlineStr">
+        <is>
+          <t>Выгрузка 9+3 от 14.10 (старая логика, как отправляли)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="46" t="inlineStr">
+        <is>
+          <t>Commercial margin (инкремент выручки без E-comm − РА и блогеры)</t>
+        </is>
+      </c>
+      <c r="B6" s="89" t="n">
+        <v>79.92599934437963</v>
+      </c>
+      <c r="C6" s="89" t="n">
+        <v>141.0704806976929</v>
+      </c>
+      <c r="D6" s="89" t="n">
+        <v>132.9730140892157</v>
+      </c>
+      <c r="E6" s="89" t="n">
+        <v>161.3072900874327</v>
+      </c>
+      <c r="F6" s="89" t="n">
+        <v>328.2615566602637</v>
+      </c>
+      <c r="G6" s="89" t="n">
+        <v>437.7610614028037</v>
+      </c>
+      <c r="H6" s="89" t="n">
+        <v>261.3663162682095</v>
+      </c>
+      <c r="I6" s="89" t="n">
+        <v>253.4120620304224</v>
+      </c>
+      <c r="J6" s="89" t="n">
+        <v>434.0875008000364</v>
+      </c>
+      <c r="K6" s="89" t="n">
+        <v>187.7060132808443</v>
+      </c>
+      <c r="L6" s="89" t="n">
+        <v>302.7226418468388</v>
+      </c>
+      <c r="M6" s="89" t="n">
+        <v>393.0673276715648</v>
+      </c>
+      <c r="N6" s="89">
+        <f>SUM(B6:M6)</f>
+        <v>3113.6612641797</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t>PEX admin</t>
+        </is>
+      </c>
+      <c r="B7" s="89" t="n">
+        <v>-92.88636049999999</v>
+      </c>
+      <c r="C7" s="89" t="n">
+        <v>-94.5925139</v>
+      </c>
+      <c r="D7" s="89" t="n">
+        <v>-95.10917844724878</v>
+      </c>
+      <c r="E7" s="89" t="n">
+        <v>-101.8822365107256</v>
+      </c>
+      <c r="F7" s="89" t="n">
+        <v>-112.4676209260646</v>
+      </c>
+      <c r="G7" s="89" t="n">
+        <v>-106.2402667461649</v>
+      </c>
+      <c r="H7" s="89" t="n">
+        <v>-101.3368353946933</v>
+      </c>
+      <c r="I7" s="89" t="n">
+        <v>-111.3047417725611</v>
+      </c>
+      <c r="J7" s="89" t="n">
+        <v>44.82120126104592</v>
+      </c>
+      <c r="K7" s="89" t="n">
+        <v>-111.5102827511398</v>
+      </c>
+      <c r="L7" s="89" t="n">
+        <v>-111.5102827511398</v>
+      </c>
+      <c r="M7" s="89" t="n">
+        <v>-111.5102827511398</v>
+      </c>
+      <c r="N7" s="89">
+        <f>SUM(B7:M7)</f>
+        <v>-1105.52940118983</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="46" t="inlineStr">
+        <is>
+          <t>PEX other</t>
+        </is>
+      </c>
+      <c r="B8" s="89" t="n">
+        <v>-3.05173</v>
+      </c>
+      <c r="C8" s="89" t="n">
+        <v>-0.442289</v>
+      </c>
+      <c r="D8" s="89" t="n">
+        <v>-1.224642702951454</v>
+      </c>
+      <c r="E8" s="89" t="n">
+        <v>-1.641531440093187</v>
+      </c>
+      <c r="F8" s="89" t="n">
+        <v>-1.239698623622975</v>
+      </c>
+      <c r="G8" s="89" t="n">
+        <v>-16.41692346736547</v>
+      </c>
+      <c r="H8" s="89" t="n">
+        <v>2.264459930033199</v>
+      </c>
+      <c r="I8" s="89" t="n">
+        <v>-3.169988265700941</v>
+      </c>
+      <c r="J8" s="89" t="n">
+        <v>-0.4110462535315827</v>
+      </c>
+      <c r="K8" s="89" t="n">
+        <v>-4.272655524947914</v>
+      </c>
+      <c r="L8" s="89" t="n">
+        <v>-4.142931662061526</v>
+      </c>
+      <c r="M8" s="89" t="n">
+        <v>-3.965340224999997</v>
+      </c>
+      <c r="N8" s="89">
+        <f>SUM(B8:M8)</f>
+        <v>-37.7143172352419</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B9" s="89" t="n">
+        <v>-28.528894</v>
+      </c>
+      <c r="C9" s="89" t="n">
+        <v>-1.745</v>
+      </c>
+      <c r="D9" s="89" t="n">
+        <v>9.53520363</v>
+      </c>
+      <c r="E9" s="89" t="n">
+        <v>-87.75989982000003</v>
+      </c>
+      <c r="F9" s="89" t="n">
+        <v>-43.87168396999997</v>
+      </c>
+      <c r="G9" s="89" t="n">
+        <v>-106.62055019</v>
+      </c>
+      <c r="H9" s="89" t="n">
+        <v>-120.26675859</v>
+      </c>
+      <c r="I9" s="89" t="n">
+        <v>-82.79719141</v>
+      </c>
+      <c r="J9" s="89" t="n">
+        <v>-105.089188</v>
+      </c>
+      <c r="K9" s="89" t="n">
+        <v>-104.6528311930226</v>
+      </c>
+      <c r="L9" s="89" t="n">
+        <v>-98.20793697621149</v>
+      </c>
+      <c r="M9" s="89" t="n">
+        <v>-111.6228575142901</v>
+      </c>
+      <c r="N9" s="89">
+        <f>SUM(B9:M9)</f>
+        <v>-881.627588033524</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="46" t="inlineStr">
+        <is>
+          <t>Consulting and insurance</t>
+        </is>
+      </c>
+      <c r="B10" s="89" t="n">
+        <v>-0.155854</v>
+      </c>
+      <c r="C10" s="89" t="n">
+        <v>-1.633817</v>
+      </c>
+      <c r="D10" s="89" t="n">
+        <v>0.77247476</v>
+      </c>
+      <c r="E10" s="89" t="n">
+        <v>-1.37120632</v>
+      </c>
+      <c r="F10" s="89" t="n">
+        <v>-2.464153540000001</v>
+      </c>
+      <c r="G10" s="89" t="n">
+        <v>-2.164074739999998</v>
+      </c>
+      <c r="H10" s="89" t="n">
+        <v>-0.9401674499999998</v>
+      </c>
+      <c r="I10" s="89" t="n">
+        <v>-0.96429323</v>
+      </c>
+      <c r="J10" s="89" t="n">
+        <v>-3.887514700000001</v>
+      </c>
+      <c r="K10" s="89" t="n">
+        <v>-1.28350724</v>
+      </c>
+      <c r="L10" s="89" t="n">
+        <v>-1.28350724</v>
+      </c>
+      <c r="M10" s="89" t="n">
+        <v>-1.28350724</v>
+      </c>
+      <c r="N10" s="89">
+        <f>SUM(B10:M10)</f>
+        <v>-16.65912794</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t>Other OPEX</t>
+        </is>
+      </c>
+      <c r="B11" s="89" t="n">
+        <v>-0.7198396500000001</v>
+      </c>
+      <c r="C11" s="89" t="n">
+        <v>-0.8385263100000001</v>
+      </c>
+      <c r="D11" s="89" t="n">
+        <v>-0.6837224500000001</v>
+      </c>
+      <c r="E11" s="89" t="n">
+        <v>-0.6697872100000001</v>
+      </c>
+      <c r="F11" s="89" t="n">
+        <v>-0.1033913200000003</v>
+      </c>
+      <c r="G11" s="89" t="n">
+        <v>-12.41837982</v>
+      </c>
+      <c r="H11" s="89" t="n">
+        <v>-4.55995586</v>
+      </c>
+      <c r="I11" s="89" t="n">
+        <v>-6.339050920000001</v>
+      </c>
+      <c r="J11" s="89" t="n">
+        <v>-9.12317528</v>
+      </c>
+      <c r="K11" s="89" t="n">
+        <v>-5.086833899412203</v>
+      </c>
+      <c r="L11" s="89" t="n">
+        <v>-5.71548470223184</v>
+      </c>
+      <c r="M11" s="89" t="n">
+        <v>-7.299500450465856</v>
+      </c>
+      <c r="N11" s="89">
+        <f>SUM(B11:M11)</f>
+        <v>-53.5576478721099</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="87" t="inlineStr">
+        <is>
+          <t>Total OPEX</t>
+        </is>
+      </c>
+      <c r="B12" s="90">
+        <f>B7+B8+B9+B10+B11</f>
+        <v>-125.34267815</v>
+      </c>
+      <c r="C12" s="90">
+        <f>C7+C8+C9+C10+C11</f>
+        <v>-99.25214621</v>
+      </c>
+      <c r="D12" s="90">
+        <f>D7+D8+D9+D10+D11</f>
+        <v>-86.7098652102003</v>
+      </c>
+      <c r="E12" s="90">
+        <f>E7+E8+E9+E10+E11</f>
+        <v>-193.324661300819</v>
+      </c>
+      <c r="F12" s="90">
+        <f>F7+F8+F9+F10+F11</f>
+        <v>-160.146548379688</v>
+      </c>
+      <c r="G12" s="90">
+        <f>G7+G8+G9+G10+G11</f>
+        <v>-243.86019496353</v>
+      </c>
+      <c r="H12" s="90">
+        <f>H7+H8+H9+H10+H11</f>
+        <v>-224.83925736466</v>
+      </c>
+      <c r="I12" s="90">
+        <f>I7+I8+I9+I10+I11</f>
+        <v>-204.575265598262</v>
+      </c>
+      <c r="J12" s="90">
+        <f>J7+J8+J9+J10+J11</f>
+        <v>-73.6897229724857</v>
+      </c>
+      <c r="K12" s="90">
+        <f>K7+K8+K9+K10+K11</f>
+        <v>-226.806110608523</v>
+      </c>
+      <c r="L12" s="90">
+        <f>L7+L8+L9+L10+L11</f>
+        <v>-220.860143331645</v>
+      </c>
+      <c r="M12" s="90">
+        <f>M7+M8+M9+M10+M11</f>
+        <v>-235.681488180896</v>
+      </c>
+      <c r="N12" s="90">
+        <f>SUM(B12:M12)</f>
+        <v>-2095.08808227071</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="87" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B13" s="90">
+        <f>B6+B12</f>
+        <v>-45.4166788056204</v>
+      </c>
+      <c r="C13" s="90">
+        <f>C6+C12</f>
+        <v>41.8183344876929</v>
+      </c>
+      <c r="D13" s="90">
+        <f>D6+D12</f>
+        <v>46.2631488790154</v>
+      </c>
+      <c r="E13" s="90">
+        <f>E6+E12</f>
+        <v>-32.0173712133861</v>
+      </c>
+      <c r="F13" s="90">
+        <f>F6+F12</f>
+        <v>168.115008280576</v>
+      </c>
+      <c r="G13" s="90">
+        <f>G6+G12</f>
+        <v>193.900866439273</v>
+      </c>
+      <c r="H13" s="90">
+        <f>H6+H12</f>
+        <v>36.5270589035494</v>
+      </c>
+      <c r="I13" s="90">
+        <f>I6+I12</f>
+        <v>48.8367964321603</v>
+      </c>
+      <c r="J13" s="90">
+        <f>J6+J12</f>
+        <v>360.397777827551</v>
+      </c>
+      <c r="K13" s="90">
+        <f>K6+K12</f>
+        <v>-39.1000973276782</v>
+      </c>
+      <c r="L13" s="90">
+        <f>L6+L12</f>
+        <v>81.8624985151942</v>
+      </c>
+      <c r="M13" s="90">
+        <f>M6+M12</f>
+        <v>157.385839490669</v>
+      </c>
+      <c r="N13" s="90">
+        <f>SUM(B13:M13)</f>
+        <v>1018.573181909</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="87" t="inlineStr">
+        <is>
+          <t>Разноска Marketing</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="46" t="inlineStr">
+        <is>
+          <t>Прочий маркетинг: PR/GR, мероприятия для партнёров, исследования, маркетинг ВГО (мастер Sep v9)</t>
+        </is>
+      </c>
+      <c r="B16" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="89" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="89" t="n">
+        <v>-0.98325</v>
+      </c>
+      <c r="F16" s="89" t="n">
+        <v>-6.53514683</v>
+      </c>
+      <c r="G16" s="89" t="n">
+        <v>-11.43475242</v>
+      </c>
+      <c r="H16" s="89" t="n">
+        <v>-2.23038929</v>
+      </c>
+      <c r="I16" s="89" t="n">
+        <v>-6.71382945</v>
+      </c>
+      <c r="J16" s="89" t="n">
+        <v>-6.40010462</v>
+      </c>
+      <c r="K16" s="89" t="n">
+        <v>-4.418658333333334</v>
+      </c>
+      <c r="L16" s="89" t="n">
+        <v>-7.118658333333334</v>
+      </c>
+      <c r="M16" s="89" t="n">
+        <v>-5.918658333333334</v>
+      </c>
+      <c r="N16" s="89">
+        <f>SUM(B16:M16)</f>
+        <v>-51.75344761</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="87" t="inlineStr">
+        <is>
+          <t>Закупка трафика (расходы на маркетинг в сети интернет) = Marketing − прочий маркетинг</t>
+        </is>
+      </c>
+      <c r="B17" s="90">
+        <f>B9-B16</f>
+        <v>-28.528894</v>
+      </c>
+      <c r="C17" s="90">
+        <f>C9-C16</f>
+        <v>-1.745</v>
+      </c>
+      <c r="D17" s="90">
+        <f>D9-D16</f>
+        <v>9.53520363</v>
+      </c>
+      <c r="E17" s="90">
+        <f>E9-E16</f>
+        <v>-86.77664982</v>
+      </c>
+      <c r="F17" s="90">
+        <f>F9-F16</f>
+        <v>-37.33653714</v>
+      </c>
+      <c r="G17" s="90">
+        <f>G9-G16</f>
+        <v>-95.18579777</v>
+      </c>
+      <c r="H17" s="90">
+        <f>H9-H16</f>
+        <v>-118.0363693</v>
+      </c>
+      <c r="I17" s="90">
+        <f>I9-I16</f>
+        <v>-76.08336196</v>
+      </c>
+      <c r="J17" s="90">
+        <f>J9-J16</f>
+        <v>-98.68908338</v>
+      </c>
+      <c r="K17" s="90">
+        <f>K9-K16</f>
+        <v>-100.234172859689</v>
+      </c>
+      <c r="L17" s="90">
+        <f>L9-L16</f>
+        <v>-91.0892786428782</v>
+      </c>
+      <c r="M17" s="90">
+        <f>M9-M16</f>
+        <v>-105.704199180957</v>
+      </c>
+      <c r="N17" s="90">
+        <f>SUM(B17:M17)</f>
+        <v>-829.874140423524</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="87" t="inlineStr">
+        <is>
+          <t>Свод 2026 в новой логике</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="87" t="inlineStr">
+        <is>
+          <t>Commercial margin = инкремент выручки − все расходы, привязанные к выручке</t>
+        </is>
+      </c>
+      <c r="B20" s="90">
+        <f>B6+B17</f>
+        <v>51.3971053443796</v>
+      </c>
+      <c r="C20" s="90">
+        <f>C6+C17</f>
+        <v>139.325480697693</v>
+      </c>
+      <c r="D20" s="90">
+        <f>D6+D17</f>
+        <v>142.508217719216</v>
+      </c>
+      <c r="E20" s="90">
+        <f>E6+E17</f>
+        <v>74.5306402674327</v>
+      </c>
+      <c r="F20" s="90">
+        <f>F6+F17</f>
+        <v>290.925019520264</v>
+      </c>
+      <c r="G20" s="90">
+        <f>G6+G17</f>
+        <v>342.575263632804</v>
+      </c>
+      <c r="H20" s="90">
+        <f>H6+H17</f>
+        <v>143.32994696821</v>
+      </c>
+      <c r="I20" s="90">
+        <f>I6+I17</f>
+        <v>177.328700070422</v>
+      </c>
+      <c r="J20" s="90">
+        <f>J6+J17</f>
+        <v>335.398417420036</v>
+      </c>
+      <c r="K20" s="90">
+        <f>K6+K17</f>
+        <v>87.471840421155</v>
+      </c>
+      <c r="L20" s="90">
+        <f>L6+L17</f>
+        <v>211.633363203961</v>
+      </c>
+      <c r="M20" s="90">
+        <f>M6+M17</f>
+        <v>287.363128490608</v>
+      </c>
+      <c r="N20" s="90">
+        <f>SUM(B20:M20)</f>
+        <v>2283.78712375618</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="46" t="inlineStr">
+        <is>
+          <t>PEX</t>
+        </is>
+      </c>
+      <c r="B21" s="89">
+        <f>B7+B8</f>
+        <v>-95.9380905</v>
+      </c>
+      <c r="C21" s="89">
+        <f>C7+C8</f>
+        <v>-95.0348029</v>
+      </c>
+      <c r="D21" s="89">
+        <f>D7+D8</f>
+        <v>-96.3338211502002</v>
+      </c>
+      <c r="E21" s="89">
+        <f>E7+E8</f>
+        <v>-103.523767950819</v>
+      </c>
+      <c r="F21" s="89">
+        <f>F7+F8</f>
+        <v>-113.707319549688</v>
+      </c>
+      <c r="G21" s="89">
+        <f>G7+G8</f>
+        <v>-122.65719021353</v>
+      </c>
+      <c r="H21" s="89">
+        <f>H7+H8</f>
+        <v>-99.0723754646601</v>
+      </c>
+      <c r="I21" s="89">
+        <f>I7+I8</f>
+        <v>-114.474730038262</v>
+      </c>
+      <c r="J21" s="89">
+        <f>J7+J8</f>
+        <v>44.4101550075143</v>
+      </c>
+      <c r="K21" s="89">
+        <f>K7+K8</f>
+        <v>-115.782938276088</v>
+      </c>
+      <c r="L21" s="89">
+        <f>L7+L8</f>
+        <v>-115.653214413201</v>
+      </c>
+      <c r="M21" s="89">
+        <f>M7+M8</f>
+        <v>-115.47562297614</v>
+      </c>
+      <c r="N21" s="89">
+        <f>SUM(B21:M21)</f>
+        <v>-1143.24371842507</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="46" t="inlineStr">
+        <is>
+          <t>Marketing (без закупки трафика)</t>
+        </is>
+      </c>
+      <c r="B22" s="89">
+        <f>B16</f>
+        <v>0</v>
+      </c>
+      <c r="C22" s="89">
+        <f>C16</f>
+        <v>0</v>
+      </c>
+      <c r="D22" s="89">
+        <f>D16</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="89">
+        <f>E16</f>
+        <v>-0.98325</v>
+      </c>
+      <c r="F22" s="89">
+        <f>F16</f>
+        <v>-6.53514683</v>
+      </c>
+      <c r="G22" s="89">
+        <f>G16</f>
+        <v>-11.43475242</v>
+      </c>
+      <c r="H22" s="89">
+        <f>H16</f>
+        <v>-2.23038929</v>
+      </c>
+      <c r="I22" s="89">
+        <f>I16</f>
+        <v>-6.71382945</v>
+      </c>
+      <c r="J22" s="89">
+        <f>J16</f>
+        <v>-6.40010462</v>
+      </c>
+      <c r="K22" s="89">
+        <f>K16</f>
+        <v>-4.41865833333333</v>
+      </c>
+      <c r="L22" s="89">
+        <f>L16</f>
+        <v>-7.11865833333333</v>
+      </c>
+      <c r="M22" s="89">
+        <f>M16</f>
+        <v>-5.91865833333333</v>
+      </c>
+      <c r="N22" s="89">
+        <f>SUM(B22:M22)</f>
+        <v>-51.75344761</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="46" t="inlineStr">
+        <is>
+          <t>NON PEX</t>
+        </is>
+      </c>
+      <c r="B23" s="89">
+        <f>B22+B10+B11</f>
+        <v>-0.87569365</v>
+      </c>
+      <c r="C23" s="89">
+        <f>C22+C10+C11</f>
+        <v>-2.47234331</v>
+      </c>
+      <c r="D23" s="89">
+        <f>D22+D10+D11</f>
+        <v>0.08875231</v>
+      </c>
+      <c r="E23" s="89">
+        <f>E22+E10+E11</f>
+        <v>-3.02424353</v>
+      </c>
+      <c r="F23" s="89">
+        <f>F22+F10+F11</f>
+        <v>-9.10269169</v>
+      </c>
+      <c r="G23" s="89">
+        <f>G22+G10+G11</f>
+        <v>-26.01720698</v>
+      </c>
+      <c r="H23" s="89">
+        <f>H22+H10+H11</f>
+        <v>-7.7305126</v>
+      </c>
+      <c r="I23" s="89">
+        <f>I22+I10+I11</f>
+        <v>-14.0171736</v>
+      </c>
+      <c r="J23" s="89">
+        <f>J22+J10+J11</f>
+        <v>-19.4107946</v>
+      </c>
+      <c r="K23" s="89">
+        <f>K22+K10+K11</f>
+        <v>-10.7889994727455</v>
+      </c>
+      <c r="L23" s="89">
+        <f>L22+L10+L11</f>
+        <v>-14.1176502755652</v>
+      </c>
+      <c r="M23" s="89">
+        <f>M22+M10+M11</f>
+        <v>-14.5016660237992</v>
+      </c>
+      <c r="N23" s="89">
+        <f>SUM(B23:M23)</f>
+        <v>-121.97022342211</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="87" t="inlineStr">
+        <is>
+          <t>Total OPEX</t>
+        </is>
+      </c>
+      <c r="B24" s="90">
+        <f>B21+B23</f>
+        <v>-96.81378415</v>
+      </c>
+      <c r="C24" s="90">
+        <f>C21+C23</f>
+        <v>-97.50714621</v>
+      </c>
+      <c r="D24" s="90">
+        <f>D21+D23</f>
+        <v>-96.2450688402002</v>
+      </c>
+      <c r="E24" s="90">
+        <f>E21+E23</f>
+        <v>-106.548011480819</v>
+      </c>
+      <c r="F24" s="90">
+        <f>F21+F23</f>
+        <v>-122.810011239688</v>
+      </c>
+      <c r="G24" s="90">
+        <f>G21+G23</f>
+        <v>-148.67439719353</v>
+      </c>
+      <c r="H24" s="90">
+        <f>H21+H23</f>
+        <v>-106.80288806466</v>
+      </c>
+      <c r="I24" s="90">
+        <f>I21+I23</f>
+        <v>-128.491903638262</v>
+      </c>
+      <c r="J24" s="90">
+        <f>J21+J23</f>
+        <v>24.9993604075143</v>
+      </c>
+      <c r="K24" s="90">
+        <f>K21+K23</f>
+        <v>-126.571937748833</v>
+      </c>
+      <c r="L24" s="90">
+        <f>L21+L23</f>
+        <v>-129.770864688767</v>
+      </c>
+      <c r="M24" s="90">
+        <f>M21+M23</f>
+        <v>-129.977288999939</v>
+      </c>
+      <c r="N24" s="90">
+        <f>SUM(B24:M24)</f>
+        <v>-1265.21394184718</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="87" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B25" s="90">
+        <f>B20+B24</f>
+        <v>-45.4166788056204</v>
+      </c>
+      <c r="C25" s="90">
+        <f>C20+C24</f>
+        <v>41.8183344876929</v>
+      </c>
+      <c r="D25" s="90">
+        <f>D20+D24</f>
+        <v>46.2631488790155</v>
+      </c>
+      <c r="E25" s="90">
+        <f>E20+E24</f>
+        <v>-32.0173712133861</v>
+      </c>
+      <c r="F25" s="90">
+        <f>F20+F24</f>
+        <v>168.115008280576</v>
+      </c>
+      <c r="G25" s="90">
+        <f>G20+G24</f>
+        <v>193.900866439273</v>
+      </c>
+      <c r="H25" s="90">
+        <f>H20+H24</f>
+        <v>36.5270589035494</v>
+      </c>
+      <c r="I25" s="90">
+        <f>I20+I24</f>
+        <v>48.8367964321604</v>
+      </c>
+      <c r="J25" s="90">
+        <f>J20+J24</f>
+        <v>360.397777827551</v>
+      </c>
+      <c r="K25" s="90">
+        <f>K20+K24</f>
+        <v>-39.1000973276782</v>
+      </c>
+      <c r="L25" s="90">
+        <f>L20+L24</f>
+        <v>81.8624985151942</v>
+      </c>
+      <c r="M25" s="90">
+        <f>M20+M24</f>
+        <v>157.385839490669</v>
+      </c>
+      <c r="N25" s="90">
+        <f>SUM(B25:M25)</f>
+        <v>1018.573181909</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="46" t="inlineStr">
+        <is>
+          <t>Проверка: EBITDA новая логика − EBITDA 9+3 (должно быть 0)</t>
+        </is>
+      </c>
+      <c r="B27" s="89">
+        <f>ROUND(B25-B13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="89">
+        <f>ROUND(C25-C13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="89">
+        <f>ROUND(D25-D13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="89">
+        <f>ROUND(E25-E13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="89">
+        <f>ROUND(F25-F13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="89">
+        <f>ROUND(G25-G13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="H27" s="89">
+        <f>ROUND(H25-H13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="I27" s="89">
+        <f>ROUND(I25-I13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="J27" s="89">
+        <f>ROUND(J25-J13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="K27" s="89">
+        <f>ROUND(K25-K13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="L27" s="89">
+        <f>ROUND(L25-L13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="M27" s="89">
+        <f>ROUND(M25-M13,6)</f>
+        <v>0</v>
+      </c>
+      <c r="N27" s="89">
+        <f>ROUND(N25-N13,6)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="46" t="inlineStr">
+        <is>
+          <t>Проверка: «Свод 2026 (новая логика)» − расчёт, EBITDA и Commercial margin (должно быть 0)</t>
+        </is>
+      </c>
+      <c r="B28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!B60/1000000-B25,6)+ROUND('Свод 2026 (новая логика)'!B16/1000000-B20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!C60/1000000-C25,6)+ROUND('Свод 2026 (новая логика)'!C16/1000000-C20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!D60/1000000-D25,6)+ROUND('Свод 2026 (новая логика)'!D16/1000000-D20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!E60/1000000-E25,6)+ROUND('Свод 2026 (новая логика)'!E16/1000000-E20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!F60/1000000-F25,6)+ROUND('Свод 2026 (новая логика)'!F16/1000000-F20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!G60/1000000-G25,6)+ROUND('Свод 2026 (новая логика)'!G16/1000000-G20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="H28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!H60/1000000-H25,6)+ROUND('Свод 2026 (новая логика)'!H16/1000000-H20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="I28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!I60/1000000-I25,6)+ROUND('Свод 2026 (новая логика)'!I16/1000000-I20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="J28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!J60/1000000-J25,6)+ROUND('Свод 2026 (новая логика)'!J16/1000000-J20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="K28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!K60/1000000-K25,6)+ROUND('Свод 2026 (новая логика)'!K16/1000000-K20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="L28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!L60/1000000-L25,6)+ROUND('Свод 2026 (новая логика)'!L16/1000000-L20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="M28" s="89">
+        <f>ROUND('Свод 2026 (новая логика)'!M60/1000000-M25,6)+ROUND('Свод 2026 (новая логика)'!M16/1000000-M20,6)</f>
+        <v>0</v>
+      </c>
+      <c r="N28" s="89">
+        <f>SUM(B28:M28)</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>